<commit_message>
Fashion Retail Sales Data Analysis Group commit
</commit_message>
<xml_diff>
--- a/Python_Projects/Fashion_Retail_Sales_Data_Analysis/2_Descriptive_Sales_Analysis/Assets/Descriptive_Sales_Analysis_Excel.xlsx
+++ b/Python_Projects/Fashion_Retail_Sales_Data_Analysis/2_Descriptive_Sales_Analysis/Assets/Descriptive_Sales_Analysis_Excel.xlsx
@@ -285,8 +285,8 @@
   <numFmts count="4">
     <numFmt numFmtId="164" formatCode="#,##0"/>
     <numFmt numFmtId="165" formatCode="0.00%"/>
-    <numFmt numFmtId="166" formatCode="$#,##0"/>
-    <numFmt numFmtId="167" formatCode="0.00"/>
+    <numFmt numFmtId="166" formatCode="0.00"/>
+    <numFmt numFmtId="167" formatCode="$#,##0"/>
   </numFmts>
   <fonts count="18">
     <font>
@@ -342,11 +342,11 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
+      <b/>
+      <sz val="11.5"/>
+      <color rgb="FFFF0000"/>
+      <name val="Consolas"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -367,13 +367,6 @@
       <sz val="11.25"/>
       <color rgb="FF000000"/>
       <name val="consolas"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11.5"/>
-      <color rgb="FFFF0000"/>
-      <name val="Consolas"/>
       <family val="2"/>
     </font>
     <font>
@@ -413,13 +406,20 @@
     </font>
     <font>
       <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color rgb="FFF1F1F1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="75">
+  <fills count="74">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -446,7 +446,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFBB4AE"/>
+        <fgColor rgb="FFFF9F9F"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -471,12 +471,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF9F9F"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -907,7 +901,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="86">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -930,13 +924,13 @@
     <xf numFmtId="165" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="justify"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="justify"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="justify"/>
+    </xf>
+    <xf numFmtId="167" fontId="8" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="justify"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="justify"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -945,46 +939,43 @@
     <xf numFmtId="165" fontId="6" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="justify"/>
     </xf>
+    <xf numFmtId="167" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="justify"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify"/>
     </xf>
-    <xf numFmtId="167" fontId="11" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify"/>
-    </xf>
-    <xf numFmtId="166" fontId="11" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="justify"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="justify"/>
-    </xf>
-    <xf numFmtId="167" fontId="14" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="justify"/>
-    </xf>
-    <xf numFmtId="166" fontId="15" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="justify"/>
-    </xf>
-    <xf numFmtId="166" fontId="16" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="justify"/>
-    </xf>
-    <xf numFmtId="166" fontId="14" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="justify"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="justify"/>
+    </xf>
+    <xf numFmtId="166" fontId="13" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="justify"/>
+    </xf>
+    <xf numFmtId="167" fontId="14" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="justify"/>
+    </xf>
+    <xf numFmtId="167" fontId="15" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="justify"/>
+    </xf>
+    <xf numFmtId="167" fontId="13" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -999,13 +990,13 @@
     <xf numFmtId="0" fontId="5" fillId="19" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="20" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="21" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="22" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="20" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="22" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="23" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1017,16 +1008,16 @@
     <xf numFmtId="0" fontId="10" fillId="25" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="26" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="27" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="26" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="27" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="28" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="29" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="29" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="30" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1038,64 +1029,64 @@
     <xf numFmtId="0" fontId="5" fillId="32" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="33" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="33" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="34" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="35" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="36" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="37" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="38" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="39" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="40" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="35" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="36" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="37" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="38" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="39" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="40" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="41" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="42" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="43" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="44" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="45" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="46" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="47" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="48" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="49" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="50" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="51" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="52" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="42" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="43" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="44" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="45" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="46" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="47" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="48" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="49" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="50" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="51" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="52" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="53" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1110,7 +1101,7 @@
     <xf numFmtId="0" fontId="10" fillId="56" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="57" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="57" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="58" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1125,25 +1116,25 @@
     <xf numFmtId="0" fontId="5" fillId="61" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="62" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="63" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="62" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="63" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="64" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="65" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="66" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="65" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="66" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="67" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="68" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="68" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="69" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1152,16 +1143,13 @@
     <xf numFmtId="0" fontId="10" fillId="70" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="71" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="72" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="71" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="72" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="73" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="74" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify"/>
     </xf>
   </cellXfs>
@@ -1546,10 +1534,17 @@
         <v>1</v>
       </c>
       <c r="E4" s="7">
-        <v>0.5205882352941177</v>
-      </c>
-      <c r="F4" s="8"/>
-      <c r="G4" s="8"/>
+        <f>C4/SUM($C$4:C$5)</f>
+        <v>0</v>
+      </c>
+      <c r="F4" s="8">
+        <f>IF(ROW()=4,"",C4-C3)</f>
+        <v>0</v>
+      </c>
+      <c r="G4" s="8">
+        <f>IF(ROW()=4,"",(C4-C3)/C3*100)</f>
+        <v>0</v>
+      </c>
       <c r="H4" s="9">
         <v>150.3276836158192</v>
       </c>
@@ -1560,10 +1555,17 @@
         <v>1</v>
       </c>
       <c r="K4" s="12">
-        <v>0.5319121289479103</v>
-      </c>
-      <c r="L4" s="8"/>
-      <c r="M4" s="8"/>
+        <f>I4/SUM(I$4:I$5)</f>
+        <v>0</v>
+      </c>
+      <c r="L4" s="13">
+        <f>IF(ROW()=4,"",H4-H3)</f>
+        <v>0</v>
+      </c>
+      <c r="M4" s="8">
+        <f>IF(ROW()=4,"",(H4-H3)/H3*100)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="5" spans="1:14">
       <c r="A5" s="3">
@@ -1575,17 +1577,20 @@
       <c r="C5" s="5">
         <v>1630</v>
       </c>
-      <c r="D5" s="13">
+      <c r="D5" s="14">
         <v>2</v>
       </c>
       <c r="E5" s="7">
-        <v>0.4794117647058824</v>
-      </c>
-      <c r="F5" s="14">
-        <v>-140</v>
-      </c>
-      <c r="G5" s="14">
-        <v>-7.909604519774016</v>
+        <f>C5/SUM($C$4:C$5)</f>
+        <v>0</v>
+      </c>
+      <c r="F5" s="8">
+        <f>IF(ROW()=4,"",C5-C4)</f>
+        <v>0</v>
+      </c>
+      <c r="G5" s="8">
+        <f>IF(ROW()=4,"",(C5-C4)/C4*100)</f>
+        <v>0</v>
       </c>
       <c r="H5" s="9">
         <v>143.6521472392638</v>
@@ -1597,55 +1602,58 @@
         <v>2</v>
       </c>
       <c r="K5" s="12">
-        <v>0.4680878710520897</v>
-      </c>
-      <c r="L5" s="16">
-        <v>-31927</v>
-      </c>
-      <c r="M5" s="14">
-        <v>-11.99902285027059</v>
+        <f>I5/SUM(I$4:I$5)</f>
+        <v>0</v>
+      </c>
+      <c r="L5" s="13">
+        <f>IF(ROW()=4,"",H5-H4)</f>
+        <v>0</v>
+      </c>
+      <c r="M5" s="8">
+        <f>IF(ROW()=4,"",(H5-H4)/H4*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:14">
       <c r="A6" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="17"/>
-      <c r="C6" s="18">
+      <c r="B6" s="16"/>
+      <c r="C6" s="17">
         <f>SUBTOTAL(9,C4:C5)</f>
         <v>0</v>
       </c>
-      <c r="D6" s="17"/>
-      <c r="E6" s="19">
+      <c r="D6" s="16"/>
+      <c r="E6" s="18">
         <f>SUBTOTAL(9,E4:E5)</f>
         <v>0</v>
       </c>
-      <c r="F6" s="20">
+      <c r="F6" s="19">
         <f>SUBTOTAL(9,F4:F5)</f>
         <v>0</v>
       </c>
-      <c r="G6" s="20">
+      <c r="G6" s="19">
         <f>SUBTOTAL(9,G4:G5)</f>
         <v>0</v>
       </c>
-      <c r="H6" s="21">
+      <c r="H6" s="20">
         <f>SUBTOTAL(9,H4:H5)</f>
         <v>0</v>
       </c>
-      <c r="I6" s="22">
+      <c r="I6" s="21">
         <f>SUBTOTAL(9,I4:I5)</f>
         <v>0</v>
       </c>
-      <c r="J6" s="17"/>
-      <c r="K6" s="19">
+      <c r="J6" s="16"/>
+      <c r="K6" s="18">
         <f>SUBTOTAL(9,K4:K5)</f>
         <v>0</v>
       </c>
-      <c r="L6" s="23">
+      <c r="L6" s="22">
         <f>SUBTOTAL(9,L4:L5)</f>
         <v>0</v>
       </c>
-      <c r="M6" s="20">
+      <c r="M6" s="19">
         <f>SUBTOTAL(9,M4:M5)</f>
         <v>0</v>
       </c>
@@ -1739,20 +1747,27 @@
       <c r="A4" s="3">
         <v>0</v>
       </c>
-      <c r="B4" s="24" t="s">
+      <c r="B4" s="23" t="s">
         <v>17</v>
       </c>
       <c r="C4" s="5">
         <v>61</v>
       </c>
-      <c r="D4" s="25">
+      <c r="D4" s="24">
         <v>7</v>
       </c>
       <c r="E4" s="7">
-        <v>0.08664772727272728</v>
-      </c>
-      <c r="F4" s="26"/>
-      <c r="G4" s="26"/>
+        <f>C4/SUM($C$4:C$13)</f>
+        <v>0</v>
+      </c>
+      <c r="F4" s="8">
+        <f>IF(ROW()=4,"",C4-C3)</f>
+        <v>0</v>
+      </c>
+      <c r="G4" s="8">
+        <f>IF(ROW()=4,"",(C4-C3)/C3*100)</f>
+        <v>0</v>
+      </c>
       <c r="H4" s="9">
         <v>297.655737704918</v>
       </c>
@@ -1763,32 +1778,42 @@
         <v>1</v>
       </c>
       <c r="K4" s="12">
-        <v>0.1305235462838494</v>
-      </c>
-      <c r="L4" s="26"/>
-      <c r="M4" s="26"/>
+        <f>I4/SUM(I$4:I$13)</f>
+        <v>0</v>
+      </c>
+      <c r="L4" s="13">
+        <f>IF(ROW()=4,"",H4-H3)</f>
+        <v>0</v>
+      </c>
+      <c r="M4" s="8">
+        <f>IF(ROW()=4,"",(H4-H3)/H3*100)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="5" spans="1:14">
       <c r="A5" s="3">
         <v>1</v>
       </c>
-      <c r="B5" s="24" t="s">
+      <c r="B5" s="23" t="s">
         <v>18</v>
       </c>
       <c r="C5" s="5">
         <v>81</v>
       </c>
-      <c r="D5" s="27">
+      <c r="D5" s="25">
         <v>3</v>
       </c>
       <c r="E5" s="7">
-        <v>0.1150568181818182</v>
-      </c>
-      <c r="F5" s="14">
-        <v>20</v>
-      </c>
-      <c r="G5" s="14">
-        <v>32.78688524590163</v>
+        <f>C5/SUM($C$4:C$13)</f>
+        <v>0</v>
+      </c>
+      <c r="F5" s="8">
+        <f>IF(ROW()=4,"",C5-C4)</f>
+        <v>0</v>
+      </c>
+      <c r="G5" s="8">
+        <f>IF(ROW()=4,"",(C5-C4)/C4*100)</f>
+        <v>0</v>
       </c>
       <c r="H5" s="9">
         <v>180.2962962962963</v>
@@ -1796,40 +1821,46 @@
       <c r="I5" s="10">
         <v>14604</v>
       </c>
-      <c r="J5" s="28">
+      <c r="J5" s="26">
         <v>2</v>
       </c>
       <c r="K5" s="12">
-        <v>0.1049824238546751</v>
-      </c>
-      <c r="L5" s="16">
-        <v>-3553</v>
-      </c>
-      <c r="M5" s="14">
-        <v>-19.56821060747921</v>
+        <f>I5/SUM(I$4:I$13)</f>
+        <v>0</v>
+      </c>
+      <c r="L5" s="13">
+        <f>IF(ROW()=4,"",H5-H4)</f>
+        <v>0</v>
+      </c>
+      <c r="M5" s="8">
+        <f>IF(ROW()=4,"",(H5-H4)/H4*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:14">
       <c r="A6" s="3">
         <v>2</v>
       </c>
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="23" t="s">
         <v>19</v>
       </c>
       <c r="C6" s="5">
         <v>87</v>
       </c>
-      <c r="D6" s="29">
+      <c r="D6" s="27">
         <v>2</v>
       </c>
       <c r="E6" s="7">
-        <v>0.1235795454545455</v>
-      </c>
-      <c r="F6" s="14">
-        <v>6</v>
-      </c>
-      <c r="G6" s="14">
-        <v>7.407407407407418</v>
+        <f>C6/SUM($C$4:C$13)</f>
+        <v>0</v>
+      </c>
+      <c r="F6" s="8">
+        <f>IF(ROW()=4,"",C6-C5)</f>
+        <v>0</v>
+      </c>
+      <c r="G6" s="8">
+        <f>IF(ROW()=4,"",(C6-C5)/C5*100)</f>
+        <v>0</v>
       </c>
       <c r="H6" s="9">
         <v>161.4252873563218</v>
@@ -1837,40 +1868,46 @@
       <c r="I6" s="10">
         <v>14044</v>
       </c>
-      <c r="J6" s="30">
+      <c r="J6" s="28">
         <v>3</v>
       </c>
       <c r="K6" s="12">
-        <v>0.1009568036575635</v>
-      </c>
-      <c r="L6" s="16">
-        <v>-560</v>
-      </c>
-      <c r="M6" s="14">
-        <v>-3.834565872363738</v>
+        <f>I6/SUM(I$4:I$13)</f>
+        <v>0</v>
+      </c>
+      <c r="L6" s="13">
+        <f>IF(ROW()=4,"",H6-H5)</f>
+        <v>0</v>
+      </c>
+      <c r="M6" s="8">
+        <f>IF(ROW()=4,"",(H6-H5)/H5*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:14">
       <c r="A7" s="3">
         <v>3</v>
       </c>
-      <c r="B7" s="24" t="s">
+      <c r="B7" s="23" t="s">
         <v>20</v>
       </c>
       <c r="C7" s="5">
         <v>58</v>
       </c>
-      <c r="D7" s="13">
+      <c r="D7" s="14">
         <v>9.5</v>
       </c>
       <c r="E7" s="7">
-        <v>0.08238636363636363</v>
-      </c>
-      <c r="F7" s="14">
-        <v>-29</v>
-      </c>
-      <c r="G7" s="14">
-        <v>-33.33333333333334</v>
+        <f>C7/SUM($C$4:C$13)</f>
+        <v>0</v>
+      </c>
+      <c r="F7" s="8">
+        <f>IF(ROW()=4,"",C7-C6)</f>
+        <v>0</v>
+      </c>
+      <c r="G7" s="8">
+        <f>IF(ROW()=4,"",(C7-C6)/C6*100)</f>
+        <v>0</v>
       </c>
       <c r="H7" s="9">
         <v>241.2931034482759</v>
@@ -1878,40 +1915,46 @@
       <c r="I7" s="10">
         <v>13995</v>
       </c>
-      <c r="J7" s="31">
+      <c r="J7" s="29">
         <v>4</v>
       </c>
       <c r="K7" s="12">
-        <v>0.1006045618903162</v>
-      </c>
-      <c r="L7" s="16">
-        <v>-49</v>
-      </c>
-      <c r="M7" s="14">
-        <v>-0.3489034463115881</v>
+        <f>I7/SUM(I$4:I$13)</f>
+        <v>0</v>
+      </c>
+      <c r="L7" s="13">
+        <f>IF(ROW()=4,"",H7-H6)</f>
+        <v>0</v>
+      </c>
+      <c r="M7" s="8">
+        <f>IF(ROW()=4,"",(H7-H6)/H6*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:14">
       <c r="A8" s="3">
         <v>4</v>
       </c>
-      <c r="B8" s="24" t="s">
+      <c r="B8" s="23" t="s">
         <v>21</v>
       </c>
       <c r="C8" s="5">
         <v>72</v>
       </c>
-      <c r="D8" s="32">
+      <c r="D8" s="30">
         <v>5</v>
       </c>
       <c r="E8" s="7">
-        <v>0.1022727272727273</v>
-      </c>
-      <c r="F8" s="14">
-        <v>14</v>
-      </c>
-      <c r="G8" s="14">
-        <v>24.13793103448276</v>
+        <f>C8/SUM($C$4:C$13)</f>
+        <v>0</v>
+      </c>
+      <c r="F8" s="8">
+        <f>IF(ROW()=4,"",C8-C7)</f>
+        <v>0</v>
+      </c>
+      <c r="G8" s="8">
+        <f>IF(ROW()=4,"",(C8-C7)/C7*100)</f>
+        <v>0</v>
       </c>
       <c r="H8" s="9">
         <v>194.3472222222222</v>
@@ -1919,40 +1962,46 @@
       <c r="I8" s="10">
         <v>13993</v>
       </c>
-      <c r="J8" s="33">
+      <c r="J8" s="31">
         <v>5</v>
       </c>
       <c r="K8" s="12">
-        <v>0.1005901846753265</v>
-      </c>
-      <c r="L8" s="16">
-        <v>-2</v>
-      </c>
-      <c r="M8" s="14">
-        <v>-0.01429081814934285</v>
+        <f>I8/SUM(I$4:I$13)</f>
+        <v>0</v>
+      </c>
+      <c r="L8" s="13">
+        <f>IF(ROW()=4,"",H8-H7)</f>
+        <v>0</v>
+      </c>
+      <c r="M8" s="8">
+        <f>IF(ROW()=4,"",(H8-H7)/H7*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:14">
       <c r="A9" s="3">
         <v>5</v>
       </c>
-      <c r="B9" s="24" t="s">
+      <c r="B9" s="23" t="s">
         <v>22</v>
       </c>
       <c r="C9" s="5">
         <v>65</v>
       </c>
-      <c r="D9" s="34">
+      <c r="D9" s="32">
         <v>6</v>
       </c>
       <c r="E9" s="7">
-        <v>0.09232954545454546</v>
-      </c>
-      <c r="F9" s="14">
-        <v>-7</v>
-      </c>
-      <c r="G9" s="14">
-        <v>-9.722222222222221</v>
+        <f>C9/SUM($C$4:C$13)</f>
+        <v>0</v>
+      </c>
+      <c r="F9" s="8">
+        <f>IF(ROW()=4,"",C9-C8)</f>
+        <v>0</v>
+      </c>
+      <c r="G9" s="8">
+        <f>IF(ROW()=4,"",(C9-C8)/C8*100)</f>
+        <v>0</v>
       </c>
       <c r="H9" s="9">
         <v>203.3846153846154</v>
@@ -1960,40 +2009,46 @@
       <c r="I9" s="10">
         <v>13220</v>
       </c>
-      <c r="J9" s="35">
+      <c r="J9" s="33">
         <v>6</v>
       </c>
       <c r="K9" s="12">
-        <v>0.09503339108181354</v>
-      </c>
-      <c r="L9" s="16">
-        <v>-773</v>
-      </c>
-      <c r="M9" s="14">
-        <v>-5.524190666761952</v>
+        <f>I9/SUM(I$4:I$13)</f>
+        <v>0</v>
+      </c>
+      <c r="L9" s="13">
+        <f>IF(ROW()=4,"",H9-H8)</f>
+        <v>0</v>
+      </c>
+      <c r="M9" s="8">
+        <f>IF(ROW()=4,"",(H9-H8)/H8*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:14">
       <c r="A10" s="3">
         <v>6</v>
       </c>
-      <c r="B10" s="24" t="s">
+      <c r="B10" s="23" t="s">
         <v>23</v>
       </c>
       <c r="C10" s="5">
         <v>59</v>
       </c>
-      <c r="D10" s="36">
+      <c r="D10" s="34">
         <v>8</v>
       </c>
       <c r="E10" s="7">
-        <v>0.08380681818181818</v>
-      </c>
-      <c r="F10" s="14">
-        <v>-6</v>
-      </c>
-      <c r="G10" s="14">
-        <v>-9.230769230769232</v>
+        <f>C10/SUM($C$4:C$13)</f>
+        <v>0</v>
+      </c>
+      <c r="F10" s="8">
+        <f>IF(ROW()=4,"",C10-C9)</f>
+        <v>0</v>
+      </c>
+      <c r="G10" s="8">
+        <f>IF(ROW()=4,"",(C10-C9)/C9*100)</f>
+        <v>0</v>
       </c>
       <c r="H10" s="9">
         <v>220.4237288135593</v>
@@ -2001,40 +2056,46 @@
       <c r="I10" s="10">
         <v>13005</v>
       </c>
-      <c r="J10" s="37">
+      <c r="J10" s="35">
         <v>7</v>
       </c>
       <c r="K10" s="12">
-        <v>0.09348784047042248</v>
-      </c>
-      <c r="L10" s="16">
-        <v>-215</v>
-      </c>
-      <c r="M10" s="14">
-        <v>-1.626323751891079</v>
+        <f>I10/SUM(I$4:I$13)</f>
+        <v>0</v>
+      </c>
+      <c r="L10" s="13">
+        <f>IF(ROW()=4,"",H10-H9)</f>
+        <v>0</v>
+      </c>
+      <c r="M10" s="8">
+        <f>IF(ROW()=4,"",(H10-H9)/H9*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:14">
       <c r="A11" s="3">
         <v>7</v>
       </c>
-      <c r="B11" s="24" t="s">
+      <c r="B11" s="23" t="s">
         <v>24</v>
       </c>
       <c r="C11" s="5">
         <v>73</v>
       </c>
-      <c r="D11" s="38">
+      <c r="D11" s="36">
         <v>4</v>
       </c>
       <c r="E11" s="7">
-        <v>0.1036931818181818</v>
-      </c>
-      <c r="F11" s="14">
-        <v>14</v>
-      </c>
-      <c r="G11" s="14">
-        <v>23.72881355932204</v>
+        <f>C11/SUM($C$4:C$13)</f>
+        <v>0</v>
+      </c>
+      <c r="F11" s="8">
+        <f>IF(ROW()=4,"",C11-C10)</f>
+        <v>0</v>
+      </c>
+      <c r="G11" s="8">
+        <f>IF(ROW()=4,"",(C11-C10)/C10*100)</f>
+        <v>0</v>
       </c>
       <c r="H11" s="9">
         <v>174.7671232876712</v>
@@ -2042,24 +2103,27 @@
       <c r="I11" s="10">
         <v>12758</v>
       </c>
-      <c r="J11" s="39">
+      <c r="J11" s="37">
         <v>8</v>
       </c>
       <c r="K11" s="12">
-        <v>0.09171225441919646</v>
-      </c>
-      <c r="L11" s="16">
-        <v>-247</v>
-      </c>
-      <c r="M11" s="14">
-        <v>-1.899269511726254</v>
+        <f>I11/SUM(I$4:I$13)</f>
+        <v>0</v>
+      </c>
+      <c r="L11" s="13">
+        <f>IF(ROW()=4,"",H11-H10)</f>
+        <v>0</v>
+      </c>
+      <c r="M11" s="8">
+        <f>IF(ROW()=4,"",(H11-H10)/H10*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:14">
       <c r="A12" s="3">
         <v>8</v>
       </c>
-      <c r="B12" s="24" t="s">
+      <c r="B12" s="23" t="s">
         <v>25</v>
       </c>
       <c r="C12" s="5">
@@ -2069,13 +2133,16 @@
         <v>1</v>
       </c>
       <c r="E12" s="7">
-        <v>0.1278409090909091</v>
-      </c>
-      <c r="F12" s="14">
-        <v>17</v>
-      </c>
-      <c r="G12" s="14">
-        <v>23.28767123287672</v>
+        <f>C12/SUM($C$4:C$13)</f>
+        <v>0</v>
+      </c>
+      <c r="F12" s="8">
+        <f>IF(ROW()=4,"",C12-C11)</f>
+        <v>0</v>
+      </c>
+      <c r="G12" s="8">
+        <f>IF(ROW()=4,"",(C12-C11)/C11*100)</f>
+        <v>0</v>
       </c>
       <c r="H12" s="9">
         <v>141.3777777777778</v>
@@ -2083,40 +2150,46 @@
       <c r="I12" s="10">
         <v>12724</v>
       </c>
-      <c r="J12" s="40">
+      <c r="J12" s="38">
         <v>9</v>
       </c>
       <c r="K12" s="12">
-        <v>0.09146784176437182</v>
-      </c>
-      <c r="L12" s="16">
-        <v>-34</v>
-      </c>
-      <c r="M12" s="14">
-        <v>-0.2664994513246643</v>
+        <f>I12/SUM(I$4:I$13)</f>
+        <v>0</v>
+      </c>
+      <c r="L12" s="13">
+        <f>IF(ROW()=4,"",H12-H11)</f>
+        <v>0</v>
+      </c>
+      <c r="M12" s="8">
+        <f>IF(ROW()=4,"",(H12-H11)/H11*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:14">
       <c r="A13" s="3">
         <v>9</v>
       </c>
-      <c r="B13" s="24" t="s">
+      <c r="B13" s="23" t="s">
         <v>26</v>
       </c>
       <c r="C13" s="5">
         <v>58</v>
       </c>
-      <c r="D13" s="13">
+      <c r="D13" s="14">
         <v>9.5</v>
       </c>
       <c r="E13" s="7">
-        <v>0.08238636363636363</v>
-      </c>
-      <c r="F13" s="14">
-        <v>-32</v>
-      </c>
-      <c r="G13" s="14">
-        <v>-35.55555555555555</v>
+        <f>C13/SUM($C$4:C$13)</f>
+        <v>0</v>
+      </c>
+      <c r="F13" s="8">
+        <f>IF(ROW()=4,"",C13-C12)</f>
+        <v>0</v>
+      </c>
+      <c r="G13" s="8">
+        <f>IF(ROW()=4,"",(C13-C12)/C12*100)</f>
+        <v>0</v>
       </c>
       <c r="H13" s="9">
         <v>217.3965517241379</v>
@@ -2128,55 +2201,58 @@
         <v>10</v>
       </c>
       <c r="K13" s="12">
-        <v>0.09064115190246497</v>
-      </c>
-      <c r="L13" s="16">
-        <v>-115</v>
-      </c>
-      <c r="M13" s="14">
-        <v>-0.9038038352719324</v>
+        <f>I13/SUM(I$4:I$13)</f>
+        <v>0</v>
+      </c>
+      <c r="L13" s="13">
+        <f>IF(ROW()=4,"",H13-H12)</f>
+        <v>0</v>
+      </c>
+      <c r="M13" s="8">
+        <f>IF(ROW()=4,"",(H13-H12)/H12*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:14">
       <c r="A14" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="17"/>
-      <c r="C14" s="18">
+      <c r="B14" s="16"/>
+      <c r="C14" s="17">
         <f>SUBTOTAL(9,C4:C13)</f>
         <v>0</v>
       </c>
-      <c r="D14" s="17"/>
-      <c r="E14" s="19">
+      <c r="D14" s="16"/>
+      <c r="E14" s="18">
         <f>SUBTOTAL(9,E4:E13)</f>
         <v>0</v>
       </c>
-      <c r="F14" s="20">
+      <c r="F14" s="19">
         <f>SUBTOTAL(9,F4:F13)</f>
         <v>0</v>
       </c>
-      <c r="G14" s="20">
+      <c r="G14" s="19">
         <f>SUBTOTAL(9,G4:G13)</f>
         <v>0</v>
       </c>
-      <c r="H14" s="21">
+      <c r="H14" s="20">
         <f>SUBTOTAL(9,H4:H13)</f>
         <v>0</v>
       </c>
-      <c r="I14" s="22">
+      <c r="I14" s="21">
         <f>SUBTOTAL(9,I4:I13)</f>
         <v>0</v>
       </c>
-      <c r="J14" s="17"/>
-      <c r="K14" s="19">
+      <c r="J14" s="16"/>
+      <c r="K14" s="18">
         <f>SUBTOTAL(9,K4:K13)</f>
         <v>0</v>
       </c>
-      <c r="L14" s="23">
+      <c r="L14" s="22">
         <f>SUBTOTAL(9,L4:L13)</f>
         <v>0</v>
       </c>
-      <c r="M14" s="20">
+      <c r="M14" s="19">
         <f>SUBTOTAL(9,M4:M13)</f>
         <v>0</v>
       </c>
@@ -2270,7 +2346,7 @@
       <c r="A4" s="3">
         <v>40</v>
       </c>
-      <c r="B4" s="24" t="s">
+      <c r="B4" s="23" t="s">
         <v>28</v>
       </c>
       <c r="C4" s="5">
@@ -2280,10 +2356,17 @@
         <v>1</v>
       </c>
       <c r="E4" s="7">
-        <v>0.1146711635750422</v>
-      </c>
-      <c r="F4" s="26"/>
-      <c r="G4" s="26"/>
+        <f>C4/SUM($C$4:C$13)</f>
+        <v>0</v>
+      </c>
+      <c r="F4" s="8">
+        <f>IF(ROW()=4,"",C4-C3)</f>
+        <v>0</v>
+      </c>
+      <c r="G4" s="8">
+        <f>IF(ROW()=4,"",(C4-C3)/C3*100)</f>
+        <v>0</v>
+      </c>
       <c r="H4" s="9">
         <v>104.9852941176471</v>
       </c>
@@ -2294,32 +2377,42 @@
         <v>1</v>
       </c>
       <c r="K4" s="12">
-        <v>0.115267865792618</v>
-      </c>
-      <c r="L4" s="26"/>
-      <c r="M4" s="26"/>
+        <f>I4/SUM(I$4:I$13)</f>
+        <v>0</v>
+      </c>
+      <c r="L4" s="13">
+        <f>IF(ROW()=4,"",H4-H3)</f>
+        <v>0</v>
+      </c>
+      <c r="M4" s="8">
+        <f>IF(ROW()=4,"",(H4-H3)/H3*100)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="5" spans="1:14">
       <c r="A5" s="3">
         <v>41</v>
       </c>
-      <c r="B5" s="24" t="s">
+      <c r="B5" s="23" t="s">
         <v>29</v>
       </c>
       <c r="C5" s="5">
         <v>59</v>
       </c>
-      <c r="D5" s="41">
+      <c r="D5" s="39">
         <v>5</v>
       </c>
       <c r="E5" s="7">
-        <v>0.09949409780775717</v>
-      </c>
-      <c r="F5" s="14">
-        <v>-9</v>
-      </c>
-      <c r="G5" s="14">
-        <v>-13.23529411764706</v>
+        <f>C5/SUM($C$4:C$13)</f>
+        <v>0</v>
+      </c>
+      <c r="F5" s="8">
+        <f>IF(ROW()=4,"",C5-C4)</f>
+        <v>0</v>
+      </c>
+      <c r="G5" s="8">
+        <f>IF(ROW()=4,"",(C5-C4)/C4*100)</f>
+        <v>0</v>
       </c>
       <c r="H5" s="9">
         <v>111.0677966101695</v>
@@ -2327,40 +2420,46 @@
       <c r="I5" s="10">
         <v>6553</v>
       </c>
-      <c r="J5" s="28">
+      <c r="J5" s="26">
         <v>2</v>
       </c>
       <c r="K5" s="12">
-        <v>0.105806180773081</v>
-      </c>
-      <c r="L5" s="16">
-        <v>-586</v>
-      </c>
-      <c r="M5" s="14">
-        <v>-8.208432553578938</v>
+        <f>I5/SUM(I$4:I$13)</f>
+        <v>0</v>
+      </c>
+      <c r="L5" s="13">
+        <f>IF(ROW()=4,"",H5-H4)</f>
+        <v>0</v>
+      </c>
+      <c r="M5" s="8">
+        <f>IF(ROW()=4,"",(H5-H4)/H4*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:14">
       <c r="A6" s="3">
         <v>42</v>
       </c>
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="23" t="s">
         <v>30</v>
       </c>
       <c r="C6" s="5">
         <v>67</v>
       </c>
-      <c r="D6" s="42">
+      <c r="D6" s="40">
         <v>2</v>
       </c>
       <c r="E6" s="7">
-        <v>0.1129848229342327</v>
-      </c>
-      <c r="F6" s="14">
-        <v>8</v>
-      </c>
-      <c r="G6" s="14">
-        <v>13.55932203389831</v>
+        <f>C6/SUM($C$4:C$13)</f>
+        <v>0</v>
+      </c>
+      <c r="F6" s="8">
+        <f>IF(ROW()=4,"",C6-C5)</f>
+        <v>0</v>
+      </c>
+      <c r="G6" s="8">
+        <f>IF(ROW()=4,"",(C6-C5)/C5*100)</f>
+        <v>0</v>
       </c>
       <c r="H6" s="9">
         <v>97.77611940298507</v>
@@ -2368,40 +2467,46 @@
       <c r="I6" s="10">
         <v>6551</v>
       </c>
-      <c r="J6" s="30">
+      <c r="J6" s="28">
         <v>3</v>
       </c>
       <c r="K6" s="12">
-        <v>0.1057738883327413</v>
-      </c>
-      <c r="L6" s="16">
-        <v>-2</v>
-      </c>
-      <c r="M6" s="14">
-        <v>-0.03052037234854144</v>
+        <f>I6/SUM(I$4:I$13)</f>
+        <v>0</v>
+      </c>
+      <c r="L6" s="13">
+        <f>IF(ROW()=4,"",H6-H5)</f>
+        <v>0</v>
+      </c>
+      <c r="M6" s="8">
+        <f>IF(ROW()=4,"",(H6-H5)/H5*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:14">
       <c r="A7" s="3">
         <v>43</v>
       </c>
-      <c r="B7" s="24" t="s">
+      <c r="B7" s="23" t="s">
         <v>31</v>
       </c>
       <c r="C7" s="5">
         <v>63</v>
       </c>
-      <c r="D7" s="43">
+      <c r="D7" s="41">
         <v>3</v>
       </c>
       <c r="E7" s="7">
-        <v>0.1062394603709949</v>
-      </c>
-      <c r="F7" s="14">
-        <v>-4</v>
-      </c>
-      <c r="G7" s="14">
-        <v>-5.970149253731338</v>
+        <f>C7/SUM($C$4:C$13)</f>
+        <v>0</v>
+      </c>
+      <c r="F7" s="8">
+        <f>IF(ROW()=4,"",C7-C6)</f>
+        <v>0</v>
+      </c>
+      <c r="G7" s="8">
+        <f>IF(ROW()=4,"",(C7-C6)/C6*100)</f>
+        <v>0</v>
       </c>
       <c r="H7" s="9">
         <v>103.4920634920635</v>
@@ -2409,40 +2514,46 @@
       <c r="I7" s="10">
         <v>6520</v>
       </c>
-      <c r="J7" s="31">
+      <c r="J7" s="29">
         <v>4</v>
       </c>
       <c r="K7" s="12">
-        <v>0.1052733555074757</v>
-      </c>
-      <c r="L7" s="16">
-        <v>-31</v>
-      </c>
-      <c r="M7" s="14">
-        <v>-0.4732101969164959</v>
+        <f>I7/SUM(I$4:I$13)</f>
+        <v>0</v>
+      </c>
+      <c r="L7" s="13">
+        <f>IF(ROW()=4,"",H7-H6)</f>
+        <v>0</v>
+      </c>
+      <c r="M7" s="8">
+        <f>IF(ROW()=4,"",(H7-H6)/H6*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:14">
       <c r="A8" s="3">
         <v>44</v>
       </c>
-      <c r="B8" s="24" t="s">
+      <c r="B8" s="23" t="s">
         <v>32</v>
       </c>
       <c r="C8" s="5">
         <v>61</v>
       </c>
-      <c r="D8" s="44">
+      <c r="D8" s="42">
         <v>4</v>
       </c>
       <c r="E8" s="7">
-        <v>0.1028667790893761</v>
-      </c>
-      <c r="F8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="G8" s="14">
-        <v>-3.174603174603174</v>
+        <f>C8/SUM($C$4:C$13)</f>
+        <v>0</v>
+      </c>
+      <c r="F8" s="8">
+        <f>IF(ROW()=4,"",C8-C7)</f>
+        <v>0</v>
+      </c>
+      <c r="G8" s="8">
+        <f>IF(ROW()=4,"",(C8-C7)/C7*100)</f>
+        <v>0</v>
       </c>
       <c r="H8" s="9">
         <v>105.4098360655738</v>
@@ -2450,40 +2561,46 @@
       <c r="I8" s="10">
         <v>6430</v>
       </c>
-      <c r="J8" s="33">
+      <c r="J8" s="31">
         <v>5</v>
       </c>
       <c r="K8" s="12">
-        <v>0.1038201956921885</v>
-      </c>
-      <c r="L8" s="16">
-        <v>-90</v>
-      </c>
-      <c r="M8" s="14">
-        <v>-1.380368098159512</v>
+        <f>I8/SUM(I$4:I$13)</f>
+        <v>0</v>
+      </c>
+      <c r="L8" s="13">
+        <f>IF(ROW()=4,"",H8-H7)</f>
+        <v>0</v>
+      </c>
+      <c r="M8" s="8">
+        <f>IF(ROW()=4,"",(H8-H7)/H7*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:14">
       <c r="A9" s="3">
         <v>45</v>
       </c>
-      <c r="B9" s="24" t="s">
+      <c r="B9" s="23" t="s">
         <v>33</v>
       </c>
       <c r="C9" s="5">
         <v>57</v>
       </c>
-      <c r="D9" s="45">
+      <c r="D9" s="43">
         <v>7</v>
       </c>
       <c r="E9" s="7">
-        <v>0.09612141652613827</v>
-      </c>
-      <c r="F9" s="14">
-        <v>-4</v>
-      </c>
-      <c r="G9" s="14">
-        <v>-6.557377049180324</v>
+        <f>C9/SUM($C$4:C$13)</f>
+        <v>0</v>
+      </c>
+      <c r="F9" s="8">
+        <f>IF(ROW()=4,"",C9-C8)</f>
+        <v>0</v>
+      </c>
+      <c r="G9" s="8">
+        <f>IF(ROW()=4,"",(C9-C8)/C8*100)</f>
+        <v>0</v>
       </c>
       <c r="H9" s="9">
         <v>111.5964912280702</v>
@@ -2491,40 +2608,46 @@
       <c r="I9" s="10">
         <v>6361</v>
       </c>
-      <c r="J9" s="35">
+      <c r="J9" s="33">
         <v>6</v>
       </c>
       <c r="K9" s="12">
-        <v>0.1027061065004682</v>
-      </c>
-      <c r="L9" s="16">
-        <v>-69</v>
-      </c>
-      <c r="M9" s="14">
-        <v>-1.073094867807156</v>
+        <f>I9/SUM(I$4:I$13)</f>
+        <v>0</v>
+      </c>
+      <c r="L9" s="13">
+        <f>IF(ROW()=4,"",H9-H8)</f>
+        <v>0</v>
+      </c>
+      <c r="M9" s="8">
+        <f>IF(ROW()=4,"",(H9-H8)/H8*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:14">
       <c r="A10" s="3">
         <v>46</v>
       </c>
-      <c r="B10" s="24" t="s">
+      <c r="B10" s="23" t="s">
         <v>34</v>
       </c>
       <c r="C10" s="5">
         <v>54</v>
       </c>
-      <c r="D10" s="46">
+      <c r="D10" s="44">
         <v>9</v>
       </c>
       <c r="E10" s="7">
-        <v>0.09106239460370995</v>
-      </c>
-      <c r="F10" s="14">
-        <v>-3</v>
-      </c>
-      <c r="G10" s="14">
-        <v>-5.263157894736848</v>
+        <f>C10/SUM($C$4:C$13)</f>
+        <v>0</v>
+      </c>
+      <c r="F10" s="8">
+        <f>IF(ROW()=4,"",C10-C9)</f>
+        <v>0</v>
+      </c>
+      <c r="G10" s="8">
+        <f>IF(ROW()=4,"",(C10-C9)/C9*100)</f>
+        <v>0</v>
       </c>
       <c r="H10" s="9">
         <v>114.3703703703704</v>
@@ -2532,40 +2655,46 @@
       <c r="I10" s="10">
         <v>6176</v>
       </c>
-      <c r="J10" s="37">
+      <c r="J10" s="35">
         <v>7</v>
       </c>
       <c r="K10" s="12">
-        <v>0.09971905576904447</v>
-      </c>
-      <c r="L10" s="16">
-        <v>-185</v>
-      </c>
-      <c r="M10" s="14">
-        <v>-2.908347744065398</v>
+        <f>I10/SUM(I$4:I$13)</f>
+        <v>0</v>
+      </c>
+      <c r="L10" s="13">
+        <f>IF(ROW()=4,"",H10-H9)</f>
+        <v>0</v>
+      </c>
+      <c r="M10" s="8">
+        <f>IF(ROW()=4,"",(H10-H9)/H9*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:14">
       <c r="A11" s="3">
         <v>47</v>
       </c>
-      <c r="B11" s="24" t="s">
+      <c r="B11" s="23" t="s">
         <v>35</v>
       </c>
       <c r="C11" s="5">
         <v>57</v>
       </c>
-      <c r="D11" s="45">
+      <c r="D11" s="43">
         <v>7</v>
       </c>
       <c r="E11" s="7">
-        <v>0.09612141652613827</v>
-      </c>
-      <c r="F11" s="14">
-        <v>3</v>
-      </c>
-      <c r="G11" s="14">
-        <v>5.555555555555558</v>
+        <f>C11/SUM($C$4:C$13)</f>
+        <v>0</v>
+      </c>
+      <c r="F11" s="8">
+        <f>IF(ROW()=4,"",C11-C10)</f>
+        <v>0</v>
+      </c>
+      <c r="G11" s="8">
+        <f>IF(ROW()=4,"",(C11-C10)/C10*100)</f>
+        <v>0</v>
       </c>
       <c r="H11" s="9">
         <v>103.4035087719298</v>
@@ -2573,39 +2702,45 @@
       <c r="I11" s="10">
         <v>5894</v>
       </c>
-      <c r="J11" s="39">
+      <c r="J11" s="37">
         <v>8</v>
       </c>
       <c r="K11" s="12">
-        <v>0.09516582168114444</v>
-      </c>
-      <c r="L11" s="16">
-        <v>-282</v>
-      </c>
-      <c r="M11" s="14">
-        <v>-4.566062176165808</v>
+        <f>I11/SUM(I$4:I$13)</f>
+        <v>0</v>
+      </c>
+      <c r="L11" s="13">
+        <f>IF(ROW()=4,"",H11-H10)</f>
+        <v>0</v>
+      </c>
+      <c r="M11" s="8">
+        <f>IF(ROW()=4,"",(H11-H10)/H10*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:14">
       <c r="A12" s="3">
         <v>48</v>
       </c>
-      <c r="B12" s="24" t="s">
+      <c r="B12" s="23" t="s">
         <v>36</v>
       </c>
       <c r="C12" s="5">
         <v>57</v>
       </c>
-      <c r="D12" s="45">
+      <c r="D12" s="43">
         <v>7</v>
       </c>
       <c r="E12" s="7">
-        <v>0.09612141652613827</v>
-      </c>
-      <c r="F12" s="14">
-        <v>0</v>
-      </c>
-      <c r="G12" s="14">
+        <f>C12/SUM($C$4:C$13)</f>
+        <v>0</v>
+      </c>
+      <c r="F12" s="8">
+        <f>IF(ROW()=4,"",C12-C11)</f>
+        <v>0</v>
+      </c>
+      <c r="G12" s="8">
+        <f>IF(ROW()=4,"",(C12-C11)/C11*100)</f>
         <v>0</v>
       </c>
       <c r="H12" s="9">
@@ -2614,40 +2749,46 @@
       <c r="I12" s="10">
         <v>5507</v>
       </c>
-      <c r="J12" s="40">
+      <c r="J12" s="38">
         <v>9</v>
       </c>
       <c r="K12" s="12">
-        <v>0.08891723447540931</v>
-      </c>
-      <c r="L12" s="16">
-        <v>-387</v>
-      </c>
-      <c r="M12" s="14">
-        <v>-6.565999321343741</v>
+        <f>I12/SUM(I$4:I$13)</f>
+        <v>0</v>
+      </c>
+      <c r="L12" s="13">
+        <f>IF(ROW()=4,"",H12-H11)</f>
+        <v>0</v>
+      </c>
+      <c r="M12" s="8">
+        <f>IF(ROW()=4,"",(H12-H11)/H11*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:14">
       <c r="A13" s="3">
         <v>49</v>
       </c>
-      <c r="B13" s="24" t="s">
+      <c r="B13" s="23" t="s">
         <v>37</v>
       </c>
       <c r="C13" s="5">
         <v>50</v>
       </c>
-      <c r="D13" s="13">
+      <c r="D13" s="14">
         <v>10</v>
       </c>
       <c r="E13" s="7">
-        <v>0.08431703204047218</v>
-      </c>
-      <c r="F13" s="14">
-        <v>-7</v>
-      </c>
-      <c r="G13" s="14">
-        <v>-12.28070175438597</v>
+        <f>C13/SUM($C$4:C$13)</f>
+        <v>0</v>
+      </c>
+      <c r="F13" s="8">
+        <f>IF(ROW()=4,"",C13-C12)</f>
+        <v>0</v>
+      </c>
+      <c r="G13" s="8">
+        <f>IF(ROW()=4,"",(C13-C12)/C12*100)</f>
+        <v>0</v>
       </c>
       <c r="H13" s="9">
         <v>96.06</v>
@@ -2659,55 +2800,58 @@
         <v>10</v>
       </c>
       <c r="K13" s="12">
-        <v>0.0775502954758291</v>
-      </c>
-      <c r="L13" s="16">
-        <v>-704</v>
-      </c>
-      <c r="M13" s="14">
-        <v>-12.78372979843835</v>
+        <f>I13/SUM(I$4:I$13)</f>
+        <v>0</v>
+      </c>
+      <c r="L13" s="13">
+        <f>IF(ROW()=4,"",H13-H12)</f>
+        <v>0</v>
+      </c>
+      <c r="M13" s="8">
+        <f>IF(ROW()=4,"",(H13-H12)/H12*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:14">
       <c r="A14" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="17"/>
-      <c r="C14" s="18">
+      <c r="B14" s="16"/>
+      <c r="C14" s="17">
         <f>SUBTOTAL(9,C4:C13)</f>
         <v>0</v>
       </c>
-      <c r="D14" s="17"/>
-      <c r="E14" s="19">
+      <c r="D14" s="16"/>
+      <c r="E14" s="18">
         <f>SUBTOTAL(9,E4:E13)</f>
         <v>0</v>
       </c>
-      <c r="F14" s="20">
+      <c r="F14" s="19">
         <f>SUBTOTAL(9,F4:F13)</f>
         <v>0</v>
       </c>
-      <c r="G14" s="20">
+      <c r="G14" s="19">
         <f>SUBTOTAL(9,G4:G13)</f>
         <v>0</v>
       </c>
-      <c r="H14" s="21">
+      <c r="H14" s="20">
         <f>SUBTOTAL(9,H4:H13)</f>
         <v>0</v>
       </c>
-      <c r="I14" s="22">
+      <c r="I14" s="21">
         <f>SUBTOTAL(9,I4:I13)</f>
         <v>0</v>
       </c>
-      <c r="J14" s="17"/>
-      <c r="K14" s="19">
+      <c r="J14" s="16"/>
+      <c r="K14" s="18">
         <f>SUBTOTAL(9,K4:K13)</f>
         <v>0</v>
       </c>
-      <c r="L14" s="23">
+      <c r="L14" s="22">
         <f>SUBTOTAL(9,L4:L13)</f>
         <v>0</v>
       </c>
-      <c r="M14" s="20">
+      <c r="M14" s="19">
         <f>SUBTOTAL(9,M4:M13)</f>
         <v>0</v>
       </c>
@@ -2801,20 +2945,27 @@
       <c r="A4" s="3">
         <v>0</v>
       </c>
-      <c r="B4" s="47">
+      <c r="B4" s="45">
         <v>1</v>
       </c>
       <c r="C4" s="5">
         <v>354</v>
       </c>
-      <c r="D4" s="48">
+      <c r="D4" s="46">
         <v>4</v>
       </c>
       <c r="E4" s="7">
-        <v>0.1041176470588235</v>
-      </c>
-      <c r="F4" s="26"/>
-      <c r="G4" s="26"/>
+        <f>C4/SUM($C$4:C$8)</f>
+        <v>0</v>
+      </c>
+      <c r="F4" s="8">
+        <f>IF(ROW()=4,"",C4-C3)</f>
+        <v>0</v>
+      </c>
+      <c r="G4" s="8">
+        <f>IF(ROW()=4,"",(C4-C3)/C3*100)</f>
+        <v>0</v>
+      </c>
       <c r="H4" s="9">
         <v>139.4265536723164</v>
       </c>
@@ -2825,16 +2976,23 @@
         <v>5</v>
       </c>
       <c r="K4" s="12">
-        <v>0.0986680207023527</v>
-      </c>
-      <c r="L4" s="26"/>
-      <c r="M4" s="26"/>
+        <f>I4/SUM(I$4:I$8)</f>
+        <v>0</v>
+      </c>
+      <c r="L4" s="13">
+        <f>IF(ROW()=4,"",H4-H3)</f>
+        <v>0</v>
+      </c>
+      <c r="M4" s="8">
+        <f>IF(ROW()=4,"",(H4-H3)/H3*100)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="5" spans="1:14">
       <c r="A5" s="3">
         <v>1</v>
       </c>
-      <c r="B5" s="49">
+      <c r="B5" s="47">
         <v>2</v>
       </c>
       <c r="C5" s="5">
@@ -2844,13 +3002,16 @@
         <v>1</v>
       </c>
       <c r="E5" s="7">
-        <v>0.2758823529411765</v>
-      </c>
-      <c r="F5" s="14">
-        <v>584</v>
-      </c>
-      <c r="G5" s="14">
-        <v>164.9717514124294</v>
+        <f>C5/SUM($C$4:C$8)</f>
+        <v>0</v>
+      </c>
+      <c r="F5" s="8">
+        <f>IF(ROW()=4,"",C5-C4)</f>
+        <v>0</v>
+      </c>
+      <c r="G5" s="8">
+        <f>IF(ROW()=4,"",(C5-C4)/C4*100)</f>
+        <v>0</v>
       </c>
       <c r="H5" s="9">
         <v>126.9573560767591</v>
@@ -2858,40 +3019,46 @@
       <c r="I5" s="10">
         <v>119086</v>
       </c>
-      <c r="J5" s="50">
+      <c r="J5" s="48">
         <v>2</v>
       </c>
       <c r="K5" s="12">
-        <v>0.2380610635443883</v>
-      </c>
-      <c r="L5" s="16">
-        <v>69729</v>
-      </c>
-      <c r="M5" s="14">
-        <v>141.2747938488968</v>
+        <f>I5/SUM(I$4:I$8)</f>
+        <v>0</v>
+      </c>
+      <c r="L5" s="13">
+        <f>IF(ROW()=4,"",H5-H4)</f>
+        <v>0</v>
+      </c>
+      <c r="M5" s="8">
+        <f>IF(ROW()=4,"",(H5-H4)/H4*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:14">
       <c r="A6" s="3">
         <v>2</v>
       </c>
-      <c r="B6" s="51">
+      <c r="B6" s="49">
         <v>3</v>
       </c>
       <c r="C6" s="5">
         <v>829</v>
       </c>
-      <c r="D6" s="52">
+      <c r="D6" s="50">
         <v>3</v>
       </c>
       <c r="E6" s="7">
-        <v>0.2438235294117647</v>
-      </c>
-      <c r="F6" s="14">
-        <v>-109</v>
-      </c>
-      <c r="G6" s="14">
-        <v>-11.62046908315565</v>
+        <f>C6/SUM($C$4:C$8)</f>
+        <v>0</v>
+      </c>
+      <c r="F6" s="8">
+        <f>IF(ROW()=4,"",C6-C5)</f>
+        <v>0</v>
+      </c>
+      <c r="G6" s="8">
+        <f>IF(ROW()=4,"",(C6-C5)/C5*100)</f>
+        <v>0</v>
       </c>
       <c r="H6" s="9">
         <v>140.0193003618818</v>
@@ -2899,40 +3066,46 @@
       <c r="I6" s="10">
         <v>116076</v>
       </c>
-      <c r="J6" s="53">
+      <c r="J6" s="51">
         <v>3</v>
       </c>
       <c r="K6" s="12">
-        <v>0.2320438675577181</v>
-      </c>
-      <c r="L6" s="16">
-        <v>-3010</v>
-      </c>
-      <c r="M6" s="14">
-        <v>-2.527585106561647</v>
+        <f>I6/SUM(I$4:I$8)</f>
+        <v>0</v>
+      </c>
+      <c r="L6" s="13">
+        <f>IF(ROW()=4,"",H6-H5)</f>
+        <v>0</v>
+      </c>
+      <c r="M6" s="8">
+        <f>IF(ROW()=4,"",(H6-H5)/H5*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:14">
       <c r="A7" s="3">
         <v>3</v>
       </c>
-      <c r="B7" s="54">
+      <c r="B7" s="52">
         <v>4</v>
       </c>
       <c r="C7" s="5">
         <v>934</v>
       </c>
-      <c r="D7" s="55">
+      <c r="D7" s="53">
         <v>2</v>
       </c>
       <c r="E7" s="7">
-        <v>0.2747058823529412</v>
-      </c>
-      <c r="F7" s="14">
-        <v>105</v>
-      </c>
-      <c r="G7" s="14">
-        <v>12.66586248492159</v>
+        <f>C7/SUM($C$4:C$8)</f>
+        <v>0</v>
+      </c>
+      <c r="F7" s="8">
+        <f>IF(ROW()=4,"",C7-C6)</f>
+        <v>0</v>
+      </c>
+      <c r="G7" s="8">
+        <f>IF(ROW()=4,"",(C7-C6)/C6*100)</f>
+        <v>0</v>
       </c>
       <c r="H7" s="9">
         <v>160.551391862955</v>
@@ -2944,36 +3117,42 @@
         <v>1</v>
       </c>
       <c r="K7" s="12">
-        <v>0.2997703070369208</v>
-      </c>
-      <c r="L7" s="16">
-        <v>33879</v>
-      </c>
-      <c r="M7" s="14">
-        <v>29.18691202315724</v>
+        <f>I7/SUM(I$4:I$8)</f>
+        <v>0</v>
+      </c>
+      <c r="L7" s="13">
+        <f>IF(ROW()=4,"",H7-H6)</f>
+        <v>0</v>
+      </c>
+      <c r="M7" s="8">
+        <f>IF(ROW()=4,"",(H7-H6)/H6*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:14">
       <c r="A8" s="3">
         <v>4</v>
       </c>
-      <c r="B8" s="56">
+      <c r="B8" s="54">
         <v>5</v>
       </c>
       <c r="C8" s="5">
         <v>345</v>
       </c>
-      <c r="D8" s="13">
+      <c r="D8" s="14">
         <v>5</v>
       </c>
       <c r="E8" s="7">
-        <v>0.1014705882352941</v>
-      </c>
-      <c r="F8" s="14">
-        <v>-589</v>
-      </c>
-      <c r="G8" s="14">
-        <v>-63.06209850107066</v>
+        <f>C8/SUM($C$4:C$8)</f>
+        <v>0</v>
+      </c>
+      <c r="F8" s="8">
+        <f>IF(ROW()=4,"",C8-C7)</f>
+        <v>0</v>
+      </c>
+      <c r="G8" s="8">
+        <f>IF(ROW()=4,"",(C8-C7)/C7*100)</f>
+        <v>0</v>
       </c>
       <c r="H8" s="9">
         <v>190.6057971014493</v>
@@ -2981,59 +3160,62 @@
       <c r="I8" s="10">
         <v>65759</v>
       </c>
-      <c r="J8" s="57">
+      <c r="J8" s="55">
         <v>4</v>
       </c>
       <c r="K8" s="12">
-        <v>0.1314567411586201</v>
-      </c>
-      <c r="L8" s="16">
-        <v>-84196</v>
-      </c>
-      <c r="M8" s="14">
-        <v>-56.14751091994265</v>
+        <f>I8/SUM(I$4:I$8)</f>
+        <v>0</v>
+      </c>
+      <c r="L8" s="13">
+        <f>IF(ROW()=4,"",H8-H7)</f>
+        <v>0</v>
+      </c>
+      <c r="M8" s="8">
+        <f>IF(ROW()=4,"",(H8-H7)/H7*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:14">
       <c r="A9" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="17"/>
-      <c r="C9" s="18">
+      <c r="B9" s="16"/>
+      <c r="C9" s="17">
         <f>SUBTOTAL(9,C4:C8)</f>
         <v>0</v>
       </c>
-      <c r="D9" s="17"/>
-      <c r="E9" s="19">
+      <c r="D9" s="16"/>
+      <c r="E9" s="18">
         <f>SUBTOTAL(9,E4:E8)</f>
         <v>0</v>
       </c>
-      <c r="F9" s="20">
+      <c r="F9" s="19">
         <f>SUBTOTAL(9,F4:F8)</f>
         <v>0</v>
       </c>
-      <c r="G9" s="20">
+      <c r="G9" s="19">
         <f>SUBTOTAL(9,G4:G8)</f>
         <v>0</v>
       </c>
-      <c r="H9" s="21">
+      <c r="H9" s="20">
         <f>SUBTOTAL(9,H4:H8)</f>
         <v>0</v>
       </c>
-      <c r="I9" s="22">
+      <c r="I9" s="21">
         <f>SUBTOTAL(9,I4:I8)</f>
         <v>0</v>
       </c>
-      <c r="J9" s="17"/>
-      <c r="K9" s="19">
+      <c r="J9" s="16"/>
+      <c r="K9" s="18">
         <f>SUBTOTAL(9,K4:K8)</f>
         <v>0</v>
       </c>
-      <c r="L9" s="23">
+      <c r="L9" s="22">
         <f>SUBTOTAL(9,L4:L8)</f>
         <v>0</v>
       </c>
-      <c r="M9" s="20">
+      <c r="M9" s="19">
         <f>SUBTOTAL(9,M4:M8)</f>
         <v>0</v>
       </c>
@@ -3127,56 +3309,73 @@
       <c r="A4" s="3">
         <v>0</v>
       </c>
-      <c r="B4" s="58" t="s">
+      <c r="B4" s="56" t="s">
         <v>42</v>
       </c>
       <c r="C4" s="5">
         <v>504</v>
       </c>
-      <c r="D4" s="59">
+      <c r="D4" s="57">
         <v>2</v>
       </c>
       <c r="E4" s="7">
-        <v>0.148235294117647</v>
-      </c>
-      <c r="F4" s="26"/>
-      <c r="G4" s="26"/>
+        <f>C4/SUM($C$4:C$10)</f>
+        <v>0</v>
+      </c>
+      <c r="F4" s="8">
+        <f>IF(ROW()=4,"",C4-C3)</f>
+        <v>0</v>
+      </c>
+      <c r="G4" s="8">
+        <f>IF(ROW()=4,"",(C4-C3)/C3*100)</f>
+        <v>0</v>
+      </c>
       <c r="H4" s="9">
         <v>147.9027777777778</v>
       </c>
       <c r="I4" s="10">
         <v>74543</v>
       </c>
-      <c r="J4" s="31">
+      <c r="J4" s="29">
         <v>3</v>
       </c>
       <c r="K4" s="12">
-        <v>0.1490165582838397</v>
-      </c>
-      <c r="L4" s="26"/>
-      <c r="M4" s="26"/>
+        <f>I4/SUM(I$4:I$10)</f>
+        <v>0</v>
+      </c>
+      <c r="L4" s="13">
+        <f>IF(ROW()=4,"",H4-H3)</f>
+        <v>0</v>
+      </c>
+      <c r="M4" s="8">
+        <f>IF(ROW()=4,"",(H4-H3)/H3*100)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="5" spans="1:14">
       <c r="A5" s="3">
         <v>1</v>
       </c>
-      <c r="B5" s="58" t="s">
+      <c r="B5" s="56" t="s">
         <v>43</v>
       </c>
       <c r="C5" s="5">
         <v>468</v>
       </c>
-      <c r="D5" s="60">
+      <c r="D5" s="58">
         <v>6</v>
       </c>
       <c r="E5" s="7">
-        <v>0.1376470588235294</v>
-      </c>
-      <c r="F5" s="14">
-        <v>-36</v>
-      </c>
-      <c r="G5" s="14">
-        <v>-7.14285714285714</v>
+        <f>C5/SUM($C$4:C$10)</f>
+        <v>0</v>
+      </c>
+      <c r="F5" s="8">
+        <f>IF(ROW()=4,"",C5-C4)</f>
+        <v>0</v>
+      </c>
+      <c r="G5" s="8">
+        <f>IF(ROW()=4,"",(C5-C4)/C4*100)</f>
+        <v>0</v>
       </c>
       <c r="H5" s="9">
         <v>152.3696581196581</v>
@@ -3184,40 +3383,46 @@
       <c r="I5" s="10">
         <v>71309</v>
       </c>
-      <c r="J5" s="53">
+      <c r="J5" s="51">
         <v>4</v>
       </c>
       <c r="K5" s="12">
-        <v>0.1425515709679289</v>
-      </c>
-      <c r="L5" s="16">
-        <v>-3234</v>
-      </c>
-      <c r="M5" s="14">
-        <v>-4.338435533852946</v>
+        <f>I5/SUM(I$4:I$10)</f>
+        <v>0</v>
+      </c>
+      <c r="L5" s="13">
+        <f>IF(ROW()=4,"",H5-H4)</f>
+        <v>0</v>
+      </c>
+      <c r="M5" s="8">
+        <f>IF(ROW()=4,"",(H5-H4)/H4*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:14">
       <c r="A6" s="3">
         <v>2</v>
       </c>
-      <c r="B6" s="58" t="s">
+      <c r="B6" s="56" t="s">
         <v>44</v>
       </c>
       <c r="C6" s="5">
         <v>461</v>
       </c>
-      <c r="D6" s="13">
+      <c r="D6" s="14">
         <v>7</v>
       </c>
       <c r="E6" s="7">
-        <v>0.1355882352941176</v>
-      </c>
-      <c r="F6" s="14">
-        <v>-7</v>
-      </c>
-      <c r="G6" s="14">
-        <v>-1.49572649572649</v>
+        <f>C6/SUM($C$4:C$10)</f>
+        <v>0</v>
+      </c>
+      <c r="F6" s="8">
+        <f>IF(ROW()=4,"",C6-C5)</f>
+        <v>0</v>
+      </c>
+      <c r="G6" s="8">
+        <f>IF(ROW()=4,"",(C6-C5)/C5*100)</f>
+        <v>0</v>
       </c>
       <c r="H6" s="9">
         <v>134.704989154013</v>
@@ -3229,20 +3434,23 @@
         <v>7</v>
       </c>
       <c r="K6" s="12">
-        <v>0.1241401506897786</v>
-      </c>
-      <c r="L6" s="16">
-        <v>-9210</v>
-      </c>
-      <c r="M6" s="14">
-        <v>-12.91562074913405</v>
+        <f>I6/SUM(I$4:I$10)</f>
+        <v>0</v>
+      </c>
+      <c r="L6" s="13">
+        <f>IF(ROW()=4,"",H6-H5)</f>
+        <v>0</v>
+      </c>
+      <c r="M6" s="8">
+        <f>IF(ROW()=4,"",(H6-H5)/H5*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:14">
       <c r="A7" s="3">
         <v>3</v>
       </c>
-      <c r="B7" s="58" t="s">
+      <c r="B7" s="56" t="s">
         <v>45</v>
       </c>
       <c r="C7" s="5">
@@ -3252,13 +3460,16 @@
         <v>1</v>
       </c>
       <c r="E7" s="7">
-        <v>0.1547058823529412</v>
-      </c>
-      <c r="F7" s="14">
-        <v>65</v>
-      </c>
-      <c r="G7" s="14">
-        <v>14.0997830802603</v>
+        <f>C7/SUM($C$4:C$10)</f>
+        <v>0</v>
+      </c>
+      <c r="F7" s="8">
+        <f>IF(ROW()=4,"",C7-C6)</f>
+        <v>0</v>
+      </c>
+      <c r="G7" s="8">
+        <f>IF(ROW()=4,"",(C7-C6)/C6*100)</f>
+        <v>0</v>
       </c>
       <c r="H7" s="9">
         <v>128.1882129277567</v>
@@ -3266,40 +3477,46 @@
       <c r="I7" s="10">
         <v>67427</v>
       </c>
-      <c r="J7" s="37">
+      <c r="J7" s="35">
         <v>5</v>
       </c>
       <c r="K7" s="12">
-        <v>0.1347911873067151</v>
-      </c>
-      <c r="L7" s="16">
-        <v>5328</v>
-      </c>
-      <c r="M7" s="14">
-        <v>8.579848306736015</v>
+        <f>I7/SUM(I$4:I$10)</f>
+        <v>0</v>
+      </c>
+      <c r="L7" s="13">
+        <f>IF(ROW()=4,"",H7-H6)</f>
+        <v>0</v>
+      </c>
+      <c r="M7" s="8">
+        <f>IF(ROW()=4,"",(H7-H6)/H6*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:14">
       <c r="A8" s="3">
         <v>4</v>
       </c>
-      <c r="B8" s="58" t="s">
+      <c r="B8" s="56" t="s">
         <v>46</v>
       </c>
       <c r="C8" s="5">
         <v>472</v>
       </c>
-      <c r="D8" s="45">
+      <c r="D8" s="43">
         <v>5</v>
       </c>
       <c r="E8" s="7">
-        <v>0.1388235294117647</v>
-      </c>
-      <c r="F8" s="14">
-        <v>-54</v>
-      </c>
-      <c r="G8" s="14">
-        <v>-10.26615969581749</v>
+        <f>C8/SUM($C$4:C$10)</f>
+        <v>0</v>
+      </c>
+      <c r="F8" s="8">
+        <f>IF(ROW()=4,"",C8-C7)</f>
+        <v>0</v>
+      </c>
+      <c r="G8" s="8">
+        <f>IF(ROW()=4,"",(C8-C7)/C7*100)</f>
+        <v>0</v>
       </c>
       <c r="H8" s="9">
         <v>167.8665254237288</v>
@@ -3307,40 +3524,46 @@
       <c r="I8" s="10">
         <v>79233</v>
       </c>
-      <c r="J8" s="61">
+      <c r="J8" s="59">
         <v>2</v>
       </c>
       <c r="K8" s="12">
-        <v>0.1583921892398142</v>
-      </c>
-      <c r="L8" s="16">
-        <v>11806</v>
-      </c>
-      <c r="M8" s="14">
-        <v>17.50930636095334</v>
+        <f>I8/SUM(I$4:I$10)</f>
+        <v>0</v>
+      </c>
+      <c r="L8" s="13">
+        <f>IF(ROW()=4,"",H8-H7)</f>
+        <v>0</v>
+      </c>
+      <c r="M8" s="8">
+        <f>IF(ROW()=4,"",(H8-H7)/H7*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:14">
       <c r="A9" s="3">
         <v>5</v>
       </c>
-      <c r="B9" s="58" t="s">
+      <c r="B9" s="56" t="s">
         <v>47</v>
       </c>
       <c r="C9" s="5">
         <v>482</v>
       </c>
-      <c r="D9" s="52">
+      <c r="D9" s="50">
         <v>4</v>
       </c>
       <c r="E9" s="7">
-        <v>0.1417647058823529</v>
-      </c>
-      <c r="F9" s="14">
-        <v>10</v>
-      </c>
-      <c r="G9" s="14">
-        <v>2.118644067796605</v>
+        <f>C9/SUM($C$4:C$10)</f>
+        <v>0</v>
+      </c>
+      <c r="F9" s="8">
+        <f>IF(ROW()=4,"",C9-C8)</f>
+        <v>0</v>
+      </c>
+      <c r="G9" s="8">
+        <f>IF(ROW()=4,"",(C9-C8)/C8*100)</f>
+        <v>0</v>
       </c>
       <c r="H9" s="9">
         <v>129.2697095435685</v>
@@ -3348,40 +3571,46 @@
       <c r="I9" s="10">
         <v>62308</v>
       </c>
-      <c r="J9" s="62">
+      <c r="J9" s="60">
         <v>6</v>
       </c>
       <c r="K9" s="12">
-        <v>0.1245579559925075</v>
-      </c>
-      <c r="L9" s="16">
-        <v>-16925</v>
-      </c>
-      <c r="M9" s="14">
-        <v>-21.36104905784206</v>
+        <f>I9/SUM(I$4:I$10)</f>
+        <v>0</v>
+      </c>
+      <c r="L9" s="13">
+        <f>IF(ROW()=4,"",H9-H8)</f>
+        <v>0</v>
+      </c>
+      <c r="M9" s="8">
+        <f>IF(ROW()=4,"",(H9-H8)/H8*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:14">
       <c r="A10" s="3">
         <v>6</v>
       </c>
-      <c r="B10" s="58" t="s">
+      <c r="B10" s="56" t="s">
         <v>48</v>
       </c>
       <c r="C10" s="5">
         <v>487</v>
       </c>
-      <c r="D10" s="44">
+      <c r="D10" s="42">
         <v>3</v>
       </c>
       <c r="E10" s="7">
-        <v>0.1432352941176471</v>
-      </c>
-      <c r="F10" s="14">
-        <v>5</v>
-      </c>
-      <c r="G10" s="14">
-        <v>1.037344398340245</v>
+        <f>C10/SUM($C$4:C$10)</f>
+        <v>0</v>
+      </c>
+      <c r="F10" s="8">
+        <f>IF(ROW()=4,"",C10-C9)</f>
+        <v>0</v>
+      </c>
+      <c r="G10" s="8">
+        <f>IF(ROW()=4,"",(C10-C9)/C9*100)</f>
+        <v>0</v>
       </c>
       <c r="H10" s="9">
         <v>171.0759753593429</v>
@@ -3393,55 +3622,58 @@
         <v>1</v>
       </c>
       <c r="K10" s="12">
-        <v>0.1665503875194159</v>
-      </c>
-      <c r="L10" s="16">
-        <v>21006</v>
-      </c>
-      <c r="M10" s="14">
-        <v>33.71316684855876</v>
+        <f>I10/SUM(I$4:I$10)</f>
+        <v>0</v>
+      </c>
+      <c r="L10" s="13">
+        <f>IF(ROW()=4,"",H10-H9)</f>
+        <v>0</v>
+      </c>
+      <c r="M10" s="8">
+        <f>IF(ROW()=4,"",(H10-H9)/H9*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:14">
       <c r="A11" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="17"/>
-      <c r="C11" s="18">
+      <c r="B11" s="16"/>
+      <c r="C11" s="17">
         <f>SUBTOTAL(9,C4:C10)</f>
         <v>0</v>
       </c>
-      <c r="D11" s="17"/>
-      <c r="E11" s="19">
+      <c r="D11" s="16"/>
+      <c r="E11" s="18">
         <f>SUBTOTAL(9,E4:E10)</f>
         <v>0</v>
       </c>
-      <c r="F11" s="20">
+      <c r="F11" s="19">
         <f>SUBTOTAL(9,F4:F10)</f>
         <v>0</v>
       </c>
-      <c r="G11" s="20">
+      <c r="G11" s="19">
         <f>SUBTOTAL(9,G4:G10)</f>
         <v>0</v>
       </c>
-      <c r="H11" s="21">
+      <c r="H11" s="20">
         <f>SUBTOTAL(9,H4:H10)</f>
         <v>0</v>
       </c>
-      <c r="I11" s="22">
+      <c r="I11" s="21">
         <f>SUBTOTAL(9,I4:I10)</f>
         <v>0</v>
       </c>
-      <c r="J11" s="17"/>
-      <c r="K11" s="19">
+      <c r="J11" s="16"/>
+      <c r="K11" s="18">
         <f>SUBTOTAL(9,K4:K10)</f>
         <v>0</v>
       </c>
-      <c r="L11" s="23">
+      <c r="L11" s="22">
         <f>SUBTOTAL(9,L4:L10)</f>
         <v>0</v>
       </c>
-      <c r="M11" s="20">
+      <c r="M11" s="19">
         <f>SUBTOTAL(9,M4:M10)</f>
         <v>0</v>
       </c>
@@ -3535,56 +3767,73 @@
       <c r="A4" s="3">
         <v>0</v>
       </c>
-      <c r="B4" s="63" t="s">
+      <c r="B4" s="61" t="s">
         <v>51</v>
       </c>
       <c r="C4" s="5">
         <v>292</v>
       </c>
-      <c r="D4" s="64">
+      <c r="D4" s="62">
         <v>7</v>
       </c>
       <c r="E4" s="7">
-        <v>0.08588235294117647</v>
-      </c>
-      <c r="F4" s="26"/>
-      <c r="G4" s="26"/>
+        <f>C4/SUM($C$4:C$15)</f>
+        <v>0</v>
+      </c>
+      <c r="F4" s="8">
+        <f>IF(ROW()=4,"",C4-C3)</f>
+        <v>0</v>
+      </c>
+      <c r="G4" s="8">
+        <f>IF(ROW()=4,"",(C4-C3)/C3*100)</f>
+        <v>0</v>
+      </c>
       <c r="H4" s="9">
         <v>122.3287671232877</v>
       </c>
       <c r="I4" s="10">
         <v>35720</v>
       </c>
-      <c r="J4" s="65">
+      <c r="J4" s="63">
         <v>11</v>
       </c>
       <c r="K4" s="12">
-        <v>0.07140672446639866</v>
-      </c>
-      <c r="L4" s="26"/>
-      <c r="M4" s="26"/>
+        <f>I4/SUM(I$4:I$15)</f>
+        <v>0</v>
+      </c>
+      <c r="L4" s="13">
+        <f>IF(ROW()=4,"",H4-H3)</f>
+        <v>0</v>
+      </c>
+      <c r="M4" s="8">
+        <f>IF(ROW()=4,"",(H4-H3)/H3*100)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="5" spans="1:14">
       <c r="A5" s="3">
         <v>1</v>
       </c>
-      <c r="B5" s="63" t="s">
+      <c r="B5" s="61" t="s">
         <v>52</v>
       </c>
       <c r="C5" s="5">
         <v>251</v>
       </c>
-      <c r="D5" s="66">
+      <c r="D5" s="64">
         <v>11</v>
       </c>
       <c r="E5" s="7">
-        <v>0.0738235294117647</v>
-      </c>
-      <c r="F5" s="14">
-        <v>-41</v>
-      </c>
-      <c r="G5" s="14">
-        <v>-14.04109589041096</v>
+        <f>C5/SUM($C$4:C$15)</f>
+        <v>0</v>
+      </c>
+      <c r="F5" s="8">
+        <f>IF(ROW()=4,"",C5-C4)</f>
+        <v>0</v>
+      </c>
+      <c r="G5" s="8">
+        <f>IF(ROW()=4,"",(C5-C4)/C4*100)</f>
+        <v>0</v>
       </c>
       <c r="H5" s="9">
         <v>158.5059760956175</v>
@@ -3592,40 +3841,46 @@
       <c r="I5" s="10">
         <v>39785</v>
       </c>
-      <c r="J5" s="67">
+      <c r="J5" s="65">
         <v>7</v>
       </c>
       <c r="K5" s="12">
-        <v>0.07953293765105461</v>
-      </c>
-      <c r="L5" s="16">
-        <v>4065</v>
-      </c>
-      <c r="M5" s="14">
-        <v>11.38017917133258</v>
+        <f>I5/SUM(I$4:I$15)</f>
+        <v>0</v>
+      </c>
+      <c r="L5" s="13">
+        <f>IF(ROW()=4,"",H5-H4)</f>
+        <v>0</v>
+      </c>
+      <c r="M5" s="8">
+        <f>IF(ROW()=4,"",(H5-H4)/H4*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:14">
       <c r="A6" s="3">
         <v>2</v>
       </c>
-      <c r="B6" s="63" t="s">
+      <c r="B6" s="61" t="s">
         <v>53</v>
       </c>
       <c r="C6" s="5">
         <v>277</v>
       </c>
-      <c r="D6" s="68">
+      <c r="D6" s="66">
         <v>8</v>
       </c>
       <c r="E6" s="7">
-        <v>0.08147058823529411</v>
-      </c>
-      <c r="F6" s="14">
-        <v>26</v>
-      </c>
-      <c r="G6" s="14">
-        <v>10.35856573705178</v>
+        <f>C6/SUM($C$4:C$15)</f>
+        <v>0</v>
+      </c>
+      <c r="F6" s="8">
+        <f>IF(ROW()=4,"",C6-C5)</f>
+        <v>0</v>
+      </c>
+      <c r="G6" s="8">
+        <f>IF(ROW()=4,"",(C6-C5)/C5*100)</f>
+        <v>0</v>
       </c>
       <c r="H6" s="9">
         <v>159.8592057761733</v>
@@ -3633,40 +3888,46 @@
       <c r="I6" s="10">
         <v>44281</v>
       </c>
-      <c r="J6" s="69">
+      <c r="J6" s="67">
         <v>4</v>
       </c>
       <c r="K6" s="12">
-        <v>0.08852074933081185</v>
-      </c>
-      <c r="L6" s="16">
-        <v>4496</v>
-      </c>
-      <c r="M6" s="14">
-        <v>11.30074148548448</v>
+        <f>I6/SUM(I$4:I$15)</f>
+        <v>0</v>
+      </c>
+      <c r="L6" s="13">
+        <f>IF(ROW()=4,"",H6-H5)</f>
+        <v>0</v>
+      </c>
+      <c r="M6" s="8">
+        <f>IF(ROW()=4,"",(H6-H5)/H5*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:14">
       <c r="A7" s="3">
         <v>3</v>
       </c>
-      <c r="B7" s="63" t="s">
+      <c r="B7" s="61" t="s">
         <v>54</v>
       </c>
       <c r="C7" s="5">
         <v>295</v>
       </c>
-      <c r="D7" s="70">
+      <c r="D7" s="68">
         <v>6</v>
       </c>
       <c r="E7" s="7">
-        <v>0.08676470588235294</v>
-      </c>
-      <c r="F7" s="14">
-        <v>18</v>
-      </c>
-      <c r="G7" s="14">
-        <v>6.498194945848379</v>
+        <f>C7/SUM($C$4:C$15)</f>
+        <v>0</v>
+      </c>
+      <c r="F7" s="8">
+        <f>IF(ROW()=4,"",C7-C6)</f>
+        <v>0</v>
+      </c>
+      <c r="G7" s="8">
+        <f>IF(ROW()=4,"",(C7-C6)/C6*100)</f>
+        <v>0</v>
       </c>
       <c r="H7" s="9">
         <v>158.6576271186441</v>
@@ -3674,40 +3935,46 @@
       <c r="I7" s="10">
         <v>46804</v>
       </c>
-      <c r="J7" s="71">
+      <c r="J7" s="69">
         <v>3</v>
       </c>
       <c r="K7" s="12">
-        <v>0.09356439899007063</v>
-      </c>
-      <c r="L7" s="16">
-        <v>2523</v>
-      </c>
-      <c r="M7" s="14">
-        <v>5.697703303900092</v>
+        <f>I7/SUM(I$4:I$15)</f>
+        <v>0</v>
+      </c>
+      <c r="L7" s="13">
+        <f>IF(ROW()=4,"",H7-H6)</f>
+        <v>0</v>
+      </c>
+      <c r="M7" s="8">
+        <f>IF(ROW()=4,"",(H7-H6)/H6*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:14">
       <c r="A8" s="3">
         <v>4</v>
       </c>
-      <c r="B8" s="63" t="s">
+      <c r="B8" s="61" t="s">
         <v>55</v>
       </c>
       <c r="C8" s="5">
         <v>308</v>
       </c>
-      <c r="D8" s="72">
+      <c r="D8" s="70">
         <v>2</v>
       </c>
       <c r="E8" s="7">
-        <v>0.09058823529411765</v>
-      </c>
-      <c r="F8" s="14">
-        <v>13</v>
-      </c>
-      <c r="G8" s="14">
-        <v>4.406779661016946</v>
+        <f>C8/SUM($C$4:C$15)</f>
+        <v>0</v>
+      </c>
+      <c r="F8" s="8">
+        <f>IF(ROW()=4,"",C8-C7)</f>
+        <v>0</v>
+      </c>
+      <c r="G8" s="8">
+        <f>IF(ROW()=4,"",(C8-C7)/C7*100)</f>
+        <v>0</v>
       </c>
       <c r="H8" s="9">
         <v>167.6590909090909</v>
@@ -3715,40 +3982,46 @@
       <c r="I8" s="10">
         <v>51639</v>
       </c>
-      <c r="J8" s="73">
+      <c r="J8" s="71">
         <v>2</v>
       </c>
       <c r="K8" s="12">
-        <v>0.103229894868991</v>
-      </c>
-      <c r="L8" s="16">
-        <v>4835</v>
-      </c>
-      <c r="M8" s="14">
-        <v>10.33031364840611</v>
+        <f>I8/SUM(I$4:I$15)</f>
+        <v>0</v>
+      </c>
+      <c r="L8" s="13">
+        <f>IF(ROW()=4,"",H8-H7)</f>
+        <v>0</v>
+      </c>
+      <c r="M8" s="8">
+        <f>IF(ROW()=4,"",(H8-H7)/H7*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:14">
       <c r="A9" s="3">
         <v>5</v>
       </c>
-      <c r="B9" s="63" t="s">
+      <c r="B9" s="61" t="s">
         <v>56</v>
       </c>
       <c r="C9" s="5">
         <v>262</v>
       </c>
-      <c r="D9" s="74">
+      <c r="D9" s="72">
         <v>9</v>
       </c>
       <c r="E9" s="7">
-        <v>0.07705882352941176</v>
-      </c>
-      <c r="F9" s="14">
-        <v>-46</v>
-      </c>
-      <c r="G9" s="14">
-        <v>-14.93506493506493</v>
+        <f>C9/SUM($C$4:C$15)</f>
+        <v>0</v>
+      </c>
+      <c r="F9" s="8">
+        <f>IF(ROW()=4,"",C9-C8)</f>
+        <v>0</v>
+      </c>
+      <c r="G9" s="8">
+        <f>IF(ROW()=4,"",(C9-C8)/C8*100)</f>
+        <v>0</v>
       </c>
       <c r="H9" s="9">
         <v>157.6145038167939</v>
@@ -3756,40 +4029,46 @@
       <c r="I9" s="10">
         <v>41295</v>
       </c>
-      <c r="J9" s="75">
+      <c r="J9" s="73">
         <v>6</v>
       </c>
       <c r="K9" s="12">
-        <v>0.08255153098656026</v>
-      </c>
-      <c r="L9" s="16">
-        <v>-10344</v>
-      </c>
-      <c r="M9" s="14">
-        <v>-20.03137163771568</v>
+        <f>I9/SUM(I$4:I$15)</f>
+        <v>0</v>
+      </c>
+      <c r="L9" s="13">
+        <f>IF(ROW()=4,"",H9-H8)</f>
+        <v>0</v>
+      </c>
+      <c r="M9" s="8">
+        <f>IF(ROW()=4,"",(H9-H8)/H8*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:14">
       <c r="A10" s="3">
         <v>6</v>
       </c>
-      <c r="B10" s="63" t="s">
+      <c r="B10" s="61" t="s">
         <v>57</v>
       </c>
       <c r="C10" s="5">
         <v>303</v>
       </c>
-      <c r="D10" s="76">
+      <c r="D10" s="74">
         <v>4</v>
       </c>
       <c r="E10" s="7">
-        <v>0.08911764705882352</v>
-      </c>
-      <c r="F10" s="14">
-        <v>41</v>
-      </c>
-      <c r="G10" s="14">
-        <v>15.64885496183206</v>
+        <f>C10/SUM($C$4:C$15)</f>
+        <v>0</v>
+      </c>
+      <c r="F10" s="8">
+        <f>IF(ROW()=4,"",C10-C9)</f>
+        <v>0</v>
+      </c>
+      <c r="G10" s="8">
+        <f>IF(ROW()=4,"",(C10-C9)/C9*100)</f>
+        <v>0</v>
       </c>
       <c r="H10" s="9">
         <v>129.1254125412541</v>
@@ -3797,40 +4076,46 @@
       <c r="I10" s="10">
         <v>39125</v>
       </c>
-      <c r="J10" s="77">
+      <c r="J10" s="75">
         <v>9</v>
       </c>
       <c r="K10" s="12">
-        <v>0.0782135524845422</v>
-      </c>
-      <c r="L10" s="16">
-        <v>-2170</v>
-      </c>
-      <c r="M10" s="14">
-        <v>-5.254873471364574</v>
+        <f>I10/SUM(I$4:I$15)</f>
+        <v>0</v>
+      </c>
+      <c r="L10" s="13">
+        <f>IF(ROW()=4,"",H10-H9)</f>
+        <v>0</v>
+      </c>
+      <c r="M10" s="8">
+        <f>IF(ROW()=4,"",(H10-H9)/H9*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:14">
       <c r="A11" s="3">
         <v>7</v>
       </c>
-      <c r="B11" s="63" t="s">
+      <c r="B11" s="61" t="s">
         <v>58</v>
       </c>
       <c r="C11" s="5">
         <v>301</v>
       </c>
-      <c r="D11" s="78">
+      <c r="D11" s="76">
         <v>5</v>
       </c>
       <c r="E11" s="7">
-        <v>0.08852941176470588</v>
-      </c>
-      <c r="F11" s="14">
-        <v>-2</v>
-      </c>
-      <c r="G11" s="14">
-        <v>-0.660066006600657</v>
+        <f>C11/SUM($C$4:C$15)</f>
+        <v>0</v>
+      </c>
+      <c r="F11" s="8">
+        <f>IF(ROW()=4,"",C11-C10)</f>
+        <v>0</v>
+      </c>
+      <c r="G11" s="8">
+        <f>IF(ROW()=4,"",(C11-C10)/C10*100)</f>
+        <v>0</v>
       </c>
       <c r="H11" s="9">
         <v>137.4817275747508</v>
@@ -3838,40 +4123,46 @@
       <c r="I11" s="10">
         <v>41382</v>
       </c>
-      <c r="J11" s="79">
+      <c r="J11" s="77">
         <v>5</v>
       </c>
       <c r="K11" s="12">
-        <v>0.08272544994032781</v>
-      </c>
-      <c r="L11" s="16">
-        <v>2257</v>
-      </c>
-      <c r="M11" s="14">
-        <v>5.76869009584664</v>
+        <f>I11/SUM(I$4:I$15)</f>
+        <v>0</v>
+      </c>
+      <c r="L11" s="13">
+        <f>IF(ROW()=4,"",H11-H10)</f>
+        <v>0</v>
+      </c>
+      <c r="M11" s="8">
+        <f>IF(ROW()=4,"",(H11-H10)/H10*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:14">
       <c r="A12" s="3">
         <v>8</v>
       </c>
-      <c r="B12" s="63" t="s">
+      <c r="B12" s="61" t="s">
         <v>59</v>
       </c>
       <c r="C12" s="5">
         <v>253</v>
       </c>
-      <c r="D12" s="80">
+      <c r="D12" s="78">
         <v>10</v>
       </c>
       <c r="E12" s="7">
-        <v>0.07441176470588236</v>
-      </c>
-      <c r="F12" s="14">
-        <v>-48</v>
-      </c>
-      <c r="G12" s="14">
-        <v>-15.9468438538206</v>
+        <f>C12/SUM($C$4:C$15)</f>
+        <v>0</v>
+      </c>
+      <c r="F12" s="8">
+        <f>IF(ROW()=4,"",C12-C11)</f>
+        <v>0</v>
+      </c>
+      <c r="G12" s="8">
+        <f>IF(ROW()=4,"",(C12-C11)/C11*100)</f>
+        <v>0</v>
       </c>
       <c r="H12" s="9">
         <v>120.4624505928854</v>
@@ -3883,20 +4174,23 @@
         <v>12</v>
       </c>
       <c r="K12" s="12">
-        <v>0.06092560866636147</v>
-      </c>
-      <c r="L12" s="16">
-        <v>-10905</v>
-      </c>
-      <c r="M12" s="14">
-        <v>-26.35203711758736</v>
+        <f>I12/SUM(I$4:I$15)</f>
+        <v>0</v>
+      </c>
+      <c r="L12" s="13">
+        <f>IF(ROW()=4,"",H12-H11)</f>
+        <v>0</v>
+      </c>
+      <c r="M12" s="8">
+        <f>IF(ROW()=4,"",(H12-H11)/H11*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:14">
       <c r="A13" s="3">
         <v>9</v>
       </c>
-      <c r="B13" s="63" t="s">
+      <c r="B13" s="61" t="s">
         <v>60</v>
       </c>
       <c r="C13" s="5">
@@ -3906,13 +4200,16 @@
         <v>1</v>
       </c>
       <c r="E13" s="7">
-        <v>0.09235294117647058</v>
-      </c>
-      <c r="F13" s="14">
-        <v>61</v>
-      </c>
-      <c r="G13" s="14">
-        <v>24.11067193675889</v>
+        <f>C13/SUM($C$4:C$15)</f>
+        <v>0</v>
+      </c>
+      <c r="F13" s="8">
+        <f>IF(ROW()=4,"",C13-C12)</f>
+        <v>0</v>
+      </c>
+      <c r="G13" s="8">
+        <f>IF(ROW()=4,"",(C13-C12)/C12*100)</f>
+        <v>0</v>
       </c>
       <c r="H13" s="9">
         <v>119.2515923566879</v>
@@ -3920,40 +4217,46 @@
       <c r="I13" s="10">
         <v>37445</v>
       </c>
-      <c r="J13" s="81">
+      <c r="J13" s="79">
         <v>10</v>
       </c>
       <c r="K13" s="12">
-        <v>0.07485511751523789</v>
-      </c>
-      <c r="L13" s="16">
-        <v>6968</v>
-      </c>
-      <c r="M13" s="14">
-        <v>22.8631426977721</v>
+        <f>I13/SUM(I$4:I$15)</f>
+        <v>0</v>
+      </c>
+      <c r="L13" s="13">
+        <f>IF(ROW()=4,"",H13-H12)</f>
+        <v>0</v>
+      </c>
+      <c r="M13" s="8">
+        <f>IF(ROW()=4,"",(H13-H12)/H12*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:14">
       <c r="A14" s="3">
         <v>10</v>
       </c>
-      <c r="B14" s="63" t="s">
+      <c r="B14" s="61" t="s">
         <v>61</v>
       </c>
       <c r="C14" s="5">
         <v>238</v>
       </c>
-      <c r="D14" s="13">
+      <c r="D14" s="14">
         <v>12</v>
       </c>
       <c r="E14" s="7">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="F14" s="14">
-        <v>-76</v>
-      </c>
-      <c r="G14" s="14">
-        <v>-24.20382165605095</v>
+        <f>C14/SUM($C$4:C$15)</f>
+        <v>0</v>
+      </c>
+      <c r="F14" s="8">
+        <f>IF(ROW()=4,"",C14-C13)</f>
+        <v>0</v>
+      </c>
+      <c r="G14" s="8">
+        <f>IF(ROW()=4,"",(C14-C13)/C13*100)</f>
+        <v>0</v>
       </c>
       <c r="H14" s="9">
         <v>165.0252100840336</v>
@@ -3961,40 +4264,46 @@
       <c r="I14" s="10">
         <v>39276</v>
       </c>
-      <c r="J14" s="82">
+      <c r="J14" s="80">
         <v>8</v>
       </c>
       <c r="K14" s="12">
-        <v>0.07851541181809277</v>
-      </c>
-      <c r="L14" s="16">
-        <v>1831</v>
-      </c>
-      <c r="M14" s="14">
-        <v>4.88983842969688</v>
+        <f>I14/SUM(I$4:I$15)</f>
+        <v>0</v>
+      </c>
+      <c r="L14" s="13">
+        <f>IF(ROW()=4,"",H14-H13)</f>
+        <v>0</v>
+      </c>
+      <c r="M14" s="8">
+        <f>IF(ROW()=4,"",(H14-H13)/H13*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:14">
       <c r="A15" s="3">
         <v>11</v>
       </c>
-      <c r="B15" s="63" t="s">
+      <c r="B15" s="61" t="s">
         <v>62</v>
       </c>
       <c r="C15" s="5">
         <v>306</v>
       </c>
-      <c r="D15" s="83">
+      <c r="D15" s="81">
         <v>3</v>
       </c>
       <c r="E15" s="7">
-        <v>0.09</v>
-      </c>
-      <c r="F15" s="14">
-        <v>68</v>
-      </c>
-      <c r="G15" s="14">
-        <v>28.57142857142858</v>
+        <f>C15/SUM($C$4:C$15)</f>
+        <v>0</v>
+      </c>
+      <c r="F15" s="8">
+        <f>IF(ROW()=4,"",C15-C14)</f>
+        <v>0</v>
+      </c>
+      <c r="G15" s="8">
+        <f>IF(ROW()=4,"",(C15-C14)/C14*100)</f>
+        <v>0</v>
       </c>
       <c r="H15" s="9">
         <v>173.2156862745098</v>
@@ -4006,55 +4315,58 @@
         <v>1</v>
       </c>
       <c r="K15" s="12">
-        <v>0.1059586232815508</v>
-      </c>
-      <c r="L15" s="16">
-        <v>13728</v>
-      </c>
-      <c r="M15" s="14">
-        <v>34.95264283531927</v>
+        <f>I15/SUM(I$4:I$15)</f>
+        <v>0</v>
+      </c>
+      <c r="L15" s="13">
+        <f>IF(ROW()=4,"",H15-H14)</f>
+        <v>0</v>
+      </c>
+      <c r="M15" s="8">
+        <f>IF(ROW()=4,"",(H15-H14)/H14*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:14">
       <c r="A16" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B16" s="17"/>
-      <c r="C16" s="18">
+      <c r="B16" s="16"/>
+      <c r="C16" s="17">
         <f>SUBTOTAL(9,C4:C15)</f>
         <v>0</v>
       </c>
-      <c r="D16" s="17"/>
-      <c r="E16" s="19">
+      <c r="D16" s="16"/>
+      <c r="E16" s="18">
         <f>SUBTOTAL(9,E4:E15)</f>
         <v>0</v>
       </c>
-      <c r="F16" s="20">
+      <c r="F16" s="19">
         <f>SUBTOTAL(9,F4:F15)</f>
         <v>0</v>
       </c>
-      <c r="G16" s="20">
+      <c r="G16" s="19">
         <f>SUBTOTAL(9,G4:G15)</f>
         <v>0</v>
       </c>
-      <c r="H16" s="21">
+      <c r="H16" s="20">
         <f>SUBTOTAL(9,H4:H15)</f>
         <v>0</v>
       </c>
-      <c r="I16" s="22">
+      <c r="I16" s="21">
         <f>SUBTOTAL(9,I4:I15)</f>
         <v>0</v>
       </c>
-      <c r="J16" s="17"/>
-      <c r="K16" s="19">
+      <c r="J16" s="16"/>
+      <c r="K16" s="18">
         <f>SUBTOTAL(9,K4:K15)</f>
         <v>0</v>
       </c>
-      <c r="L16" s="23">
+      <c r="L16" s="22">
         <f>SUBTOTAL(9,L4:L15)</f>
         <v>0</v>
       </c>
-      <c r="M16" s="20">
+      <c r="M16" s="19">
         <f>SUBTOTAL(9,M4:M15)</f>
         <v>0</v>
       </c>
@@ -4148,56 +4460,73 @@
       <c r="A4" s="3">
         <v>0</v>
       </c>
-      <c r="B4" s="84" t="s">
+      <c r="B4" s="82" t="s">
         <v>65</v>
       </c>
       <c r="C4" s="5">
         <v>853</v>
       </c>
-      <c r="D4" s="52">
+      <c r="D4" s="50">
         <v>3</v>
       </c>
       <c r="E4" s="7">
-        <v>0.2508823529411764</v>
-      </c>
-      <c r="F4" s="26"/>
-      <c r="G4" s="26"/>
+        <f>C4/SUM($C$4:C$8)</f>
+        <v>0</v>
+      </c>
+      <c r="F4" s="8">
+        <f>IF(ROW()=4,"",C4-C3)</f>
+        <v>0</v>
+      </c>
+      <c r="G4" s="8">
+        <f>IF(ROW()=4,"",(C4-C3)/C3*100)</f>
+        <v>0</v>
+      </c>
       <c r="H4" s="9">
         <v>151.5849941383353</v>
       </c>
       <c r="I4" s="10">
         <v>129302</v>
       </c>
-      <c r="J4" s="50">
+      <c r="J4" s="48">
         <v>2</v>
       </c>
       <c r="K4" s="12">
-        <v>0.258483546667253</v>
-      </c>
-      <c r="L4" s="26"/>
-      <c r="M4" s="26"/>
+        <f>I4/SUM(I$4:I$8)</f>
+        <v>0</v>
+      </c>
+      <c r="L4" s="13">
+        <f>IF(ROW()=4,"",H4-H3)</f>
+        <v>0</v>
+      </c>
+      <c r="M4" s="8">
+        <f>IF(ROW()=4,"",(H4-H3)/H3*100)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="5" spans="1:14">
       <c r="A5" s="3">
         <v>1</v>
       </c>
-      <c r="B5" s="84" t="s">
+      <c r="B5" s="82" t="s">
         <v>66</v>
       </c>
       <c r="C5" s="5">
         <v>820</v>
       </c>
-      <c r="D5" s="48">
+      <c r="D5" s="46">
         <v>4</v>
       </c>
       <c r="E5" s="7">
-        <v>0.2411764705882353</v>
-      </c>
-      <c r="F5" s="14">
-        <v>-33</v>
-      </c>
-      <c r="G5" s="14">
-        <v>-3.86869871043376</v>
+        <f>C5/SUM($C$4:C$8)</f>
+        <v>0</v>
+      </c>
+      <c r="F5" s="8">
+        <f>IF(ROW()=4,"",C5-C4)</f>
+        <v>0</v>
+      </c>
+      <c r="G5" s="8">
+        <f>IF(ROW()=4,"",(C5-C4)/C4*100)</f>
+        <v>0</v>
       </c>
       <c r="H5" s="9">
         <v>146.0804878048781</v>
@@ -4205,24 +4534,27 @@
       <c r="I5" s="10">
         <v>119786</v>
       </c>
-      <c r="J5" s="53">
+      <c r="J5" s="51">
         <v>3</v>
       </c>
       <c r="K5" s="12">
-        <v>0.2394604114482651</v>
-      </c>
-      <c r="L5" s="16">
-        <v>-9516</v>
-      </c>
-      <c r="M5" s="14">
-        <v>-7.359514934030409</v>
+        <f>I5/SUM(I$4:I$8)</f>
+        <v>0</v>
+      </c>
+      <c r="L5" s="13">
+        <f>IF(ROW()=4,"",H5-H4)</f>
+        <v>0</v>
+      </c>
+      <c r="M5" s="8">
+        <f>IF(ROW()=4,"",(H5-H4)/H4*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:14">
       <c r="A6" s="3">
         <v>2</v>
       </c>
-      <c r="B6" s="84" t="s">
+      <c r="B6" s="82" t="s">
         <v>67</v>
       </c>
       <c r="C6" s="5">
@@ -4232,13 +4564,16 @@
         <v>1</v>
       </c>
       <c r="E6" s="7">
-        <v>0.2544117647058823</v>
-      </c>
-      <c r="F6" s="14">
-        <v>45</v>
-      </c>
-      <c r="G6" s="14">
-        <v>5.487804878048785</v>
+        <f>C6/SUM($C$4:C$8)</f>
+        <v>0</v>
+      </c>
+      <c r="F6" s="8">
+        <f>IF(ROW()=4,"",C6-C5)</f>
+        <v>0</v>
+      </c>
+      <c r="G6" s="8">
+        <f>IF(ROW()=4,"",(C6-C5)/C5*100)</f>
+        <v>0</v>
       </c>
       <c r="H6" s="9">
         <v>161.5468208092485</v>
@@ -4250,36 +4585,42 @@
         <v>1</v>
       </c>
       <c r="K6" s="12">
-        <v>0.2793458248456219</v>
-      </c>
-      <c r="L6" s="16">
-        <v>19952</v>
-      </c>
-      <c r="M6" s="14">
-        <v>16.6563705274406</v>
+        <f>I6/SUM(I$4:I$8)</f>
+        <v>0</v>
+      </c>
+      <c r="L6" s="13">
+        <f>IF(ROW()=4,"",H6-H5)</f>
+        <v>0</v>
+      </c>
+      <c r="M6" s="8">
+        <f>IF(ROW()=4,"",(H6-H5)/H5*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:14">
       <c r="A7" s="3">
         <v>3</v>
       </c>
-      <c r="B7" s="84" t="s">
+      <c r="B7" s="82" t="s">
         <v>68</v>
       </c>
       <c r="C7" s="5">
         <v>857</v>
       </c>
-      <c r="D7" s="55">
+      <c r="D7" s="53">
         <v>2</v>
       </c>
       <c r="E7" s="7">
-        <v>0.2520588235294118</v>
-      </c>
-      <c r="F7" s="14">
-        <v>-8</v>
-      </c>
-      <c r="G7" s="14">
-        <v>-0.9248554913294793</v>
+        <f>C7/SUM($C$4:C$8)</f>
+        <v>0</v>
+      </c>
+      <c r="F7" s="8">
+        <f>IF(ROW()=4,"",C7-C6)</f>
+        <v>0</v>
+      </c>
+      <c r="G7" s="8">
+        <f>IF(ROW()=4,"",(C7-C6)/C6*100)</f>
+        <v>0</v>
       </c>
       <c r="H7" s="9">
         <v>129.5029171528588</v>
@@ -4287,40 +4628,46 @@
       <c r="I7" s="10">
         <v>110984</v>
       </c>
-      <c r="J7" s="57">
+      <c r="J7" s="55">
         <v>4</v>
       </c>
       <c r="K7" s="12">
-        <v>0.2218646110912315</v>
-      </c>
-      <c r="L7" s="16">
-        <v>-28754</v>
-      </c>
-      <c r="M7" s="14">
-        <v>-20.5770799639325</v>
+        <f>I7/SUM(I$4:I$8)</f>
+        <v>0</v>
+      </c>
+      <c r="L7" s="13">
+        <f>IF(ROW()=4,"",H7-H6)</f>
+        <v>0</v>
+      </c>
+      <c r="M7" s="8">
+        <f>IF(ROW()=4,"",(H7-H6)/H6*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:14">
       <c r="A8" s="3">
         <v>4</v>
       </c>
-      <c r="B8" s="84" t="s">
+      <c r="B8" s="82" t="s">
         <v>69</v>
       </c>
       <c r="C8" s="5">
         <v>5</v>
       </c>
-      <c r="D8" s="13">
+      <c r="D8" s="14">
         <v>5</v>
       </c>
       <c r="E8" s="7">
-        <v>0.001470588235294118</v>
-      </c>
-      <c r="F8" s="14">
-        <v>-852</v>
-      </c>
-      <c r="G8" s="14">
-        <v>-99.41656942823805</v>
+        <f>C8/SUM($C$4:C$8)</f>
+        <v>0</v>
+      </c>
+      <c r="F8" s="8">
+        <f>IF(ROW()=4,"",C8-C7)</f>
+        <v>0</v>
+      </c>
+      <c r="G8" s="8">
+        <f>IF(ROW()=4,"",(C8-C7)/C7*100)</f>
+        <v>0</v>
       </c>
       <c r="H8" s="9">
         <v>84.59999999999999</v>
@@ -4332,55 +4679,58 @@
         <v>5</v>
       </c>
       <c r="K8" s="12">
-        <v>0.0008456059476284051</v>
-      </c>
-      <c r="L8" s="16">
-        <v>-110561</v>
-      </c>
-      <c r="M8" s="14">
-        <v>-99.61886398039357</v>
+        <f>I8/SUM(I$4:I$8)</f>
+        <v>0</v>
+      </c>
+      <c r="L8" s="13">
+        <f>IF(ROW()=4,"",H8-H7)</f>
+        <v>0</v>
+      </c>
+      <c r="M8" s="8">
+        <f>IF(ROW()=4,"",(H8-H7)/H7*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:14">
       <c r="A9" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="17"/>
-      <c r="C9" s="18">
+      <c r="B9" s="16"/>
+      <c r="C9" s="17">
         <f>SUBTOTAL(9,C4:C8)</f>
         <v>0</v>
       </c>
-      <c r="D9" s="17"/>
-      <c r="E9" s="19">
+      <c r="D9" s="16"/>
+      <c r="E9" s="18">
         <f>SUBTOTAL(9,E4:E8)</f>
         <v>0</v>
       </c>
-      <c r="F9" s="20">
+      <c r="F9" s="19">
         <f>SUBTOTAL(9,F4:F8)</f>
         <v>0</v>
       </c>
-      <c r="G9" s="20">
+      <c r="G9" s="19">
         <f>SUBTOTAL(9,G4:G8)</f>
         <v>0</v>
       </c>
-      <c r="H9" s="21">
+      <c r="H9" s="20">
         <f>SUBTOTAL(9,H4:H8)</f>
         <v>0</v>
       </c>
-      <c r="I9" s="22">
+      <c r="I9" s="21">
         <f>SUBTOTAL(9,I4:I8)</f>
         <v>0</v>
       </c>
-      <c r="J9" s="17"/>
-      <c r="K9" s="19">
+      <c r="J9" s="16"/>
+      <c r="K9" s="18">
         <f>SUBTOTAL(9,K4:K8)</f>
         <v>0</v>
       </c>
-      <c r="L9" s="23">
+      <c r="L9" s="22">
         <f>SUBTOTAL(9,L4:L8)</f>
         <v>0</v>
       </c>
-      <c r="M9" s="20">
+      <c r="M9" s="19">
         <f>SUBTOTAL(9,M4:M8)</f>
         <v>0</v>
       </c>
@@ -4474,40 +4824,54 @@
       <c r="A4" s="3">
         <v>0</v>
       </c>
-      <c r="B4" s="84" t="s">
+      <c r="B4" s="82" t="s">
         <v>72</v>
       </c>
       <c r="C4" s="5">
         <v>820</v>
       </c>
-      <c r="D4" s="13">
+      <c r="D4" s="14">
         <v>4</v>
       </c>
       <c r="E4" s="7">
-        <v>0.2411764705882353</v>
-      </c>
-      <c r="F4" s="26"/>
-      <c r="G4" s="26"/>
+        <f>C4/SUM($C$4:C$7)</f>
+        <v>0</v>
+      </c>
+      <c r="F4" s="8">
+        <f>IF(ROW()=4,"",C4-C3)</f>
+        <v>0</v>
+      </c>
+      <c r="G4" s="8">
+        <f>IF(ROW()=4,"",(C4-C3)/C3*100)</f>
+        <v>0</v>
+      </c>
       <c r="H4" s="9">
         <v>146.0804878048781</v>
       </c>
       <c r="I4" s="10">
         <v>119786</v>
       </c>
-      <c r="J4" s="37">
+      <c r="J4" s="35">
         <v>3</v>
       </c>
       <c r="K4" s="12">
-        <v>0.2394604114482651</v>
-      </c>
-      <c r="L4" s="26"/>
-      <c r="M4" s="26"/>
+        <f>I4/SUM(I$4:I$7)</f>
+        <v>0</v>
+      </c>
+      <c r="L4" s="13">
+        <f>IF(ROW()=4,"",H4-H3)</f>
+        <v>0</v>
+      </c>
+      <c r="M4" s="8">
+        <f>IF(ROW()=4,"",(H4-H3)/H3*100)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="5" spans="1:14">
       <c r="A5" s="3">
         <v>1</v>
       </c>
-      <c r="B5" s="84" t="s">
+      <c r="B5" s="82" t="s">
         <v>73</v>
       </c>
       <c r="C5" s="5">
@@ -4517,13 +4881,16 @@
         <v>1</v>
       </c>
       <c r="E5" s="7">
-        <v>0.2544117647058823</v>
-      </c>
-      <c r="F5" s="14">
-        <v>45</v>
-      </c>
-      <c r="G5" s="14">
-        <v>5.487804878048785</v>
+        <f>C5/SUM($C$4:C$7)</f>
+        <v>0</v>
+      </c>
+      <c r="F5" s="8">
+        <f>IF(ROW()=4,"",C5-C4)</f>
+        <v>0</v>
+      </c>
+      <c r="G5" s="8">
+        <f>IF(ROW()=4,"",(C5-C4)/C4*100)</f>
+        <v>0</v>
       </c>
       <c r="H5" s="9">
         <v>161.5468208092485</v>
@@ -4535,36 +4902,42 @@
         <v>1</v>
       </c>
       <c r="K5" s="12">
-        <v>0.2793458248456219</v>
-      </c>
-      <c r="L5" s="16">
-        <v>19952</v>
-      </c>
-      <c r="M5" s="14">
-        <v>16.6563705274406</v>
+        <f>I5/SUM(I$4:I$7)</f>
+        <v>0</v>
+      </c>
+      <c r="L5" s="13">
+        <f>IF(ROW()=4,"",H5-H4)</f>
+        <v>0</v>
+      </c>
+      <c r="M5" s="8">
+        <f>IF(ROW()=4,"",(H5-H4)/H4*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:14">
       <c r="A6" s="3">
         <v>2</v>
       </c>
-      <c r="B6" s="84" t="s">
+      <c r="B6" s="82" t="s">
         <v>74</v>
       </c>
       <c r="C6" s="5">
         <v>857</v>
       </c>
-      <c r="D6" s="45">
+      <c r="D6" s="43">
         <v>3</v>
       </c>
       <c r="E6" s="7">
-        <v>0.2520588235294118</v>
-      </c>
-      <c r="F6" s="14">
-        <v>-8</v>
-      </c>
-      <c r="G6" s="14">
-        <v>-0.9248554913294793</v>
+        <f>C6/SUM($C$4:C$7)</f>
+        <v>0</v>
+      </c>
+      <c r="F6" s="8">
+        <f>IF(ROW()=4,"",C6-C5)</f>
+        <v>0</v>
+      </c>
+      <c r="G6" s="8">
+        <f>IF(ROW()=4,"",(C6-C5)/C5*100)</f>
+        <v>0</v>
       </c>
       <c r="H6" s="9">
         <v>129.5029171528588</v>
@@ -4576,36 +4949,42 @@
         <v>4</v>
       </c>
       <c r="K6" s="12">
-        <v>0.2218646110912315</v>
-      </c>
-      <c r="L6" s="16">
-        <v>-28754</v>
-      </c>
-      <c r="M6" s="14">
-        <v>-20.5770799639325</v>
+        <f>I6/SUM(I$4:I$7)</f>
+        <v>0</v>
+      </c>
+      <c r="L6" s="13">
+        <f>IF(ROW()=4,"",H6-H5)</f>
+        <v>0</v>
+      </c>
+      <c r="M6" s="8">
+        <f>IF(ROW()=4,"",(H6-H5)/H5*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:14">
       <c r="A7" s="3">
         <v>3</v>
       </c>
-      <c r="B7" s="84" t="s">
+      <c r="B7" s="82" t="s">
         <v>75</v>
       </c>
       <c r="C7" s="5">
         <v>858</v>
       </c>
-      <c r="D7" s="44">
+      <c r="D7" s="42">
         <v>2</v>
       </c>
       <c r="E7" s="7">
-        <v>0.2523529411764706</v>
-      </c>
-      <c r="F7" s="14">
-        <v>1</v>
-      </c>
-      <c r="G7" s="14">
-        <v>0.1166861143523823</v>
+        <f>C7/SUM($C$4:C$7)</f>
+        <v>0</v>
+      </c>
+      <c r="F7" s="8">
+        <f>IF(ROW()=4,"",C7-C6)</f>
+        <v>0</v>
+      </c>
+      <c r="G7" s="8">
+        <f>IF(ROW()=4,"",(C7-C6)/C6*100)</f>
+        <v>0</v>
       </c>
       <c r="H7" s="9">
         <v>151.1946386946387</v>
@@ -4613,59 +4992,62 @@
       <c r="I7" s="10">
         <v>129725</v>
       </c>
-      <c r="J7" s="31">
+      <c r="J7" s="29">
         <v>2</v>
       </c>
       <c r="K7" s="12">
-        <v>0.2593291526148815</v>
-      </c>
-      <c r="L7" s="16">
-        <v>18741</v>
-      </c>
-      <c r="M7" s="14">
-        <v>16.88621783320119</v>
+        <f>I7/SUM(I$4:I$7)</f>
+        <v>0</v>
+      </c>
+      <c r="L7" s="13">
+        <f>IF(ROW()=4,"",H7-H6)</f>
+        <v>0</v>
+      </c>
+      <c r="M7" s="8">
+        <f>IF(ROW()=4,"",(H7-H6)/H6*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:14">
       <c r="A8" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="17"/>
-      <c r="C8" s="18">
+      <c r="B8" s="16"/>
+      <c r="C8" s="17">
         <f>SUBTOTAL(9,C4:C7)</f>
         <v>0</v>
       </c>
-      <c r="D8" s="17"/>
-      <c r="E8" s="19">
+      <c r="D8" s="16"/>
+      <c r="E8" s="18">
         <f>SUBTOTAL(9,E4:E7)</f>
         <v>0</v>
       </c>
-      <c r="F8" s="20">
+      <c r="F8" s="19">
         <f>SUBTOTAL(9,F4:F7)</f>
         <v>0</v>
       </c>
-      <c r="G8" s="20">
+      <c r="G8" s="19">
         <f>SUBTOTAL(9,G4:G7)</f>
         <v>0</v>
       </c>
-      <c r="H8" s="21">
+      <c r="H8" s="20">
         <f>SUBTOTAL(9,H4:H7)</f>
         <v>0</v>
       </c>
-      <c r="I8" s="22">
+      <c r="I8" s="21">
         <f>SUBTOTAL(9,I4:I7)</f>
         <v>0</v>
       </c>
-      <c r="J8" s="17"/>
-      <c r="K8" s="19">
+      <c r="J8" s="16"/>
+      <c r="K8" s="18">
         <f>SUBTOTAL(9,K4:K7)</f>
         <v>0</v>
       </c>
-      <c r="L8" s="23">
+      <c r="L8" s="22">
         <f>SUBTOTAL(9,L4:L7)</f>
         <v>0</v>
       </c>
-      <c r="M8" s="20">
+      <c r="M8" s="19">
         <f>SUBTOTAL(9,M4:M7)</f>
         <v>0</v>
       </c>
@@ -4757,20 +5139,27 @@
       <c r="A4" s="3">
         <v>0</v>
       </c>
-      <c r="B4" s="85" t="s">
+      <c r="B4" s="83" t="s">
         <v>78</v>
       </c>
       <c r="C4" s="5">
         <v>853</v>
       </c>
-      <c r="D4" s="13">
+      <c r="D4" s="14">
         <v>2</v>
       </c>
       <c r="E4" s="7">
-        <v>0.2508823529411764</v>
-      </c>
-      <c r="F4" s="8"/>
-      <c r="G4" s="8"/>
+        <f>C4/SUM($C$4:C$5)</f>
+        <v>0</v>
+      </c>
+      <c r="F4" s="8">
+        <f>IF(ROW()=4,"",C4-C3)</f>
+        <v>0</v>
+      </c>
+      <c r="G4" s="8">
+        <f>IF(ROW()=4,"",(C4-C3)/C3*100)</f>
+        <v>0</v>
+      </c>
       <c r="H4" s="9">
         <v>151.5849941383353</v>
       </c>
@@ -4781,16 +5170,23 @@
         <v>2</v>
       </c>
       <c r="K4" s="12">
-        <v>0.258483546667253</v>
-      </c>
-      <c r="L4" s="8"/>
-      <c r="M4" s="8"/>
+        <f>I4/SUM(I$4:I$5)</f>
+        <v>0</v>
+      </c>
+      <c r="L4" s="13">
+        <f>IF(ROW()=4,"",H4-H3)</f>
+        <v>0</v>
+      </c>
+      <c r="M4" s="8">
+        <f>IF(ROW()=4,"",(H4-H3)/H3*100)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="5" spans="1:14">
       <c r="A5" s="3">
         <v>1</v>
       </c>
-      <c r="B5" s="85" t="s">
+      <c r="B5" s="83" t="s">
         <v>79</v>
       </c>
       <c r="C5" s="5">
@@ -4800,13 +5196,16 @@
         <v>1</v>
       </c>
       <c r="E5" s="7">
-        <v>0.7491176470588236</v>
-      </c>
-      <c r="F5" s="14">
-        <v>1694</v>
-      </c>
-      <c r="G5" s="14">
-        <v>198.5932004689332</v>
+        <f>C5/SUM($C$4:C$5)</f>
+        <v>0</v>
+      </c>
+      <c r="F5" s="8">
+        <f>IF(ROW()=4,"",C5-C4)</f>
+        <v>0</v>
+      </c>
+      <c r="G5" s="8">
+        <f>IF(ROW()=4,"",(C5-C4)/C4*100)</f>
+        <v>0</v>
       </c>
       <c r="H5" s="9">
         <v>145.6344719277581</v>
@@ -4818,55 +5217,58 @@
         <v>1</v>
       </c>
       <c r="K5" s="12">
-        <v>0.741516453332747</v>
-      </c>
-      <c r="L5" s="16">
-        <v>241629</v>
-      </c>
-      <c r="M5" s="14">
-        <v>186.8718194614159</v>
+        <f>I5/SUM(I$4:I$5)</f>
+        <v>0</v>
+      </c>
+      <c r="L5" s="13">
+        <f>IF(ROW()=4,"",H5-H4)</f>
+        <v>0</v>
+      </c>
+      <c r="M5" s="8">
+        <f>IF(ROW()=4,"",(H5-H4)/H4*100)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:14">
       <c r="A6" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="17"/>
-      <c r="C6" s="18">
+      <c r="B6" s="16"/>
+      <c r="C6" s="17">
         <f>SUBTOTAL(9,C4:C5)</f>
         <v>0</v>
       </c>
-      <c r="D6" s="17"/>
-      <c r="E6" s="19">
+      <c r="D6" s="16"/>
+      <c r="E6" s="18">
         <f>SUBTOTAL(9,E4:E5)</f>
         <v>0</v>
       </c>
-      <c r="F6" s="20">
+      <c r="F6" s="19">
         <f>SUBTOTAL(9,F4:F5)</f>
         <v>0</v>
       </c>
-      <c r="G6" s="20">
+      <c r="G6" s="19">
         <f>SUBTOTAL(9,G4:G5)</f>
         <v>0</v>
       </c>
-      <c r="H6" s="21">
+      <c r="H6" s="20">
         <f>SUBTOTAL(9,H4:H5)</f>
         <v>0</v>
       </c>
-      <c r="I6" s="22">
+      <c r="I6" s="21">
         <f>SUBTOTAL(9,I4:I5)</f>
         <v>0</v>
       </c>
-      <c r="J6" s="17"/>
-      <c r="K6" s="19">
+      <c r="J6" s="16"/>
+      <c r="K6" s="18">
         <f>SUBTOTAL(9,K4:K5)</f>
         <v>0</v>
       </c>
-      <c r="L6" s="23">
+      <c r="L6" s="22">
         <f>SUBTOTAL(9,L4:L5)</f>
         <v>0</v>
       </c>
-      <c r="M6" s="20">
+      <c r="M6" s="19">
         <f>SUBTOTAL(9,M4:M5)</f>
         <v>0</v>
       </c>

</xml_diff>